<commit_message>
Updated Acceptance Test Plan
</commit_message>
<xml_diff>
--- a/etc/Acceptance Test Plan.xlsx
+++ b/etc/Acceptance Test Plan.xlsx
@@ -1,23 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29429"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phine\OneDrive\code2\swen\project\team-project-2251-swen-261-05-2-goated\etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5FFEAC6-C211-44AE-8625-32BFAE2EA8AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="176" documentId="13_ncr:1_{F5FFEAC6-C211-44AE-8625-32BFAE2EA8AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED661D65-0336-4FFE-9C3E-1505B0C15FDC}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Test Plan" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="140000" concurrentCalc="0"/>
+  <calcPr calcId="191028" concurrentCalc="0"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -26,33 +40,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="104">
   <si>
     <t>Instructions</t>
-  </si>
-  <si>
-    <t>Team Name</t>
-  </si>
-  <si>
-    <t>Testing Team Name</t>
-  </si>
-  <si>
-    <t>User Story</t>
-  </si>
-  <si>
-    <t>Acceptance Criterion</t>
-  </si>
-  <si>
-    <t>Sprint 3</t>
-  </si>
-  <si>
-    <t>Sprint 2</t>
-  </si>
-  <si>
-    <t>Tester initials; date; comments (required if test failed)</t>
-  </si>
-  <si>
-    <t>fill in when doing cross-team testing</t>
   </si>
   <si>
     <t>Enter your team name as specified in the cell below. When doing cross-team acceptance testing, enter the name for the testing group.
@@ -63,45 +53,81 @@
 Submit this file per the instructions specified for the sprint submissions and cross-team testing.</t>
   </si>
   <si>
+    <t>Team Name</t>
+  </si>
+  <si>
+    <t>2251-swen-261-02-goated</t>
+  </si>
+  <si>
+    <t>Testing Team Name</t>
+  </si>
+  <si>
+    <t>fill in when doing cross-team testing</t>
+  </si>
+  <si>
+    <t>User Story</t>
+  </si>
+  <si>
+    <t>Acceptance Criterion</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>Tester initials; date; comments (required if test failed)</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>As a HELPER I want to update my username so that I can my preferred name can be stored in the system.</t>
+  </si>
+  <si>
     <t>**Given** I am a Helper **when** I press the update username button **then** a modal should appear to change my username</t>
   </si>
   <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>AF, 10/21/2025</t>
+  </si>
+  <si>
     <t>**Given** I am a Manager **when** I go to the Accounts Tab **then** nothing should appear (Specifically, a "change username" button should not appear.)</t>
   </si>
   <si>
+    <t>As a USER I want to update my password so that I can keep my account secure.</t>
+  </si>
+  <si>
     <t>**Given** I am a User **when** I press the update password button **then** a modal should appear to change my password</t>
   </si>
   <si>
+    <t>As a HELPER I want to delete my account so that I can choose to no longer support or provide needs to this group.</t>
+  </si>
+  <si>
     <t>**Given** I am a Helper **when** I press the delete account button **then** my account should be deleted (after confirmation)</t>
   </si>
   <si>
     <t>**Given** I am a Manager **when** I go to the Accounts Tab **then** I should not see the delete account button</t>
   </si>
   <si>
-    <t>As a HELPER I want to delete my account so that I can choose to no longer support or provide needs to this group.</t>
-  </si>
-  <si>
-    <t>As a USER I want to update my password so that I can keep my account secure.</t>
-  </si>
-  <si>
-    <t>As a HELPER I want to update my username so that I can my preferred name can be stored in the system.</t>
-  </si>
-  <si>
     <t>As a User I want to be able to search all needs so that I can refine what I am looking to fund.</t>
   </si>
   <si>
     <t>**Given** I am a User **when** I type in the search needs box **then** the list of needs on my screen should be filtered by matching what was typed in the search box</t>
   </si>
   <si>
+    <t>As a Manager, I want to delete a need so that needs that do not need to be fulfilled can be removed from the helpers' view.</t>
+  </si>
+  <si>
     <t>**Given** I have a need that still exists and I am a manager **when** I press the delete button **then** the need should be deleted</t>
   </si>
   <si>
+    <t>AF, 10/21/2025. There is no exclusively "delete" button, but a need can be deleted by removing the name via the "Edit/Delete" button.</t>
+  </si>
+  <si>
     <t>**Given** I am a helper **when** I go to the Needs Tab **then** the delete button should not appear</t>
   </si>
   <si>
-    <t>As a Manager, I want to delete a need so that needs that do not need to be fulfilled can be removed from the helpers' view.</t>
-  </si>
-  <si>
     <t>As an accountless user I want to Create an Account so that I can log in and contribute to needs.</t>
   </si>
   <si>
@@ -126,6 +152,9 @@
     <t>Given I am a manger, When I click on a needs edit button, Then the needs edit modal should appear</t>
   </si>
   <si>
+    <t>AF, 10/21/2025. Again, this is done with the "Edit/Delete" button.</t>
+  </si>
+  <si>
     <t>Given I am a helper, When I go to the Needs Tab **then** the edit needs button should not appear</t>
   </si>
   <si>
@@ -147,12 +176,21 @@
     <t>**Given** a need is currently in my basket and I am a helper **when** press the Add to Basket button **then** nothing should change</t>
   </si>
   <si>
+    <t>**Given** I am a manager **when** go to the page that has the Add to Basket buttons (the Needs tab) **then** I should not see them</t>
+  </si>
+  <si>
     <t>As a HELPER I want to BE ABLE TO VIEW MY BASKET so that I CAN SEE WHAT I AM FUNDING.</t>
   </si>
   <si>
     <t>**Given** that I am logged in as a manager **when** I open my tabs **then** I expect a basket tab to not appear.</t>
   </si>
   <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>AF, 10/21/2025. The Basket tab is visible, though clicking it will instead return the user to the Cupboard page, no matter where the user was before.</t>
+  </si>
+  <si>
     <t>Given that I am a helper and there are no needs in my basket, When i click on my basket, there will be no needs displayed</t>
   </si>
   <si>
@@ -177,13 +215,25 @@
     <t>**Given** there are no Needs in my Basket **when** I try to remove a Need **then** I should receive an error.</t>
   </si>
   <si>
+    <t>AF, 10/21/2025. It is impossible to receive an error this way as needs can not be removed if your basket is empty.</t>
+  </si>
+  <si>
+    <t>As a USER I want to be able to log in so that I can access my account and make the changes I want to make.</t>
+  </si>
+  <si>
     <t>**Given** I am not logged in, **when** I view the home page **then** I expect to see a button which allows me to view the log-in menu.</t>
   </si>
   <si>
+    <t>AF, 10/21/2025. A homepage has not been created, with the website instead sending you directly to the login page if you are not logged in.</t>
+  </si>
+  <si>
+    <t>RL, 11/5/2025</t>
+  </si>
+  <si>
     <t>**Given** I am logged in, **when** I view the home page **then** I expect to see a button which allows me to view the needs page using my current saved login.</t>
   </si>
   <si>
-    <t>As a USER I want to be able to log in so that I can access my account and make the changes I want to make.</t>
+    <t>AF, 10/21/2025. A homepage has not been created, with the website instead sending you directly to the cupboard page if you are logged in.</t>
   </si>
   <si>
     <t>As a USER I want to be able to log out so that others cannot access my account after I make the changes I want to make.</t>
@@ -192,44 +242,128 @@
     <t>Given that I am logged in, when I view the Accounts page I should see a button to log out of my account. (It is not possible to view the Accounts page when logged out.)</t>
   </si>
   <si>
-    <t>2251-swen-261-02-goated</t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>AF, 10/21/2025</t>
-  </si>
-  <si>
-    <t>Fail</t>
-  </si>
-  <si>
-    <t>AF, 10/21/2025. A homepage has not been created, with the website instead sending you directly to the login page if you are not logged in.</t>
-  </si>
-  <si>
-    <t>AF, 10/21/2025. A homepage has not been created, with the website instead sending you directly to the cupboard page if you are logged in.</t>
-  </si>
-  <si>
-    <t>**Given** I am a manager **when** go to the page that has the Add to Basket buttons (the Needs tab) **then** I should not see them</t>
-  </si>
-  <si>
-    <t>AF, 10/21/2025. It is impossible to receive an error this way as needs can not be removed if your basket is empty.</t>
-  </si>
-  <si>
-    <t>AF, 10/21/2025. There is no exclusively "delete" button, but a need can be deleted by removing the name via the "Edit/Delete" button.</t>
-  </si>
-  <si>
-    <t>AF, 10/21/2025. Again, this is done with the "Edit/Delete" button.</t>
-  </si>
-  <si>
-    <t>AF, 10/21/2025. The Basket tab is visible, though clicking it will instead return the user to the Cupboard page, no matter where the user was before.</t>
+    <t>As a Developer, I want to be able to get the list of users who have satisfied the most points so that the information can be displayed to the user.</t>
+  </si>
+  <si>
+    <t>Given there are users who have satisfied needs in the system, when a request is made to get the top n users who contributed the most then it should return this list and a status code of 200 (OK).</t>
+  </si>
+  <si>
+    <t>Given there are no users who have satisfied needs in the system, when a request is made to get the top n users who contributed the most then it should return an empty list and a status code of 200 (OK).</t>
+  </si>
+  <si>
+    <t>As a manager I want to be able to ban a user so that they cannot do anything anymore.</t>
+  </si>
+  <si>
+    <t>**Given** I am a manager and the user is not already banned **when** I press the ban button next to the users username **then** that user should be banned</t>
+  </si>
+  <si>
+    <t>**Given** I am a manager and the user is already banned **when** I go to the users tab **then** the button should say unban user.</t>
+  </si>
+  <si>
+    <t>As a manager I want to be able to unban a user so that they can have access to the app again.</t>
+  </si>
+  <si>
+    <t>**Given** I am a manager and the user is already banned **when** I press the unban button next to the users username **then** that user should be unbanned</t>
+  </si>
+  <si>
+    <t>**Given** I am a manager and the user is not already banned **when** I go to the users tab **then** the button should say ban user.</t>
+  </si>
+  <si>
+    <t>As a Developer I want to sessions to expire so that users are automatically logged out.</t>
+  </si>
+  <si>
+    <t>**Given** I have logged in within the last hour **when** I interact with the API **then** everything works as intended</t>
+  </si>
+  <si>
+    <t>**Given** I logged in over an hour ago **when** I interact with the API **then** I should be automatically logged out</t>
+  </si>
+  <si>
+    <t>As a Developer I want to make the search feature case insensitive so that searching is more user friendly.</t>
+  </si>
+  <si>
+    <t>**Given** I type something into the search bar **when** I enter the search **then** it provides results regardless of capitalization.</t>
+  </si>
+  <si>
+    <t>As a Developer, I want to be able to get the list of most recently satisfied needs so that the data can be displayed to the user.</t>
+  </si>
+  <si>
+    <t>Given there are satisfied needs in the system, when a request is made to get the n most recent satisfied needs then it should return this list and a status code of 200 (OK).</t>
+  </si>
+  <si>
+    <t>Given there are no satisfied needs in the system, when a request is made to get the n most recent satisfied needs then it should return an empty list and a status code of 200 (OK).</t>
+  </si>
+  <si>
+    <t>As a banned user I want to not have access to any site features except login, logout, viewing needs, searching needs, and deleting my account so that my ban has an effect</t>
+  </si>
+  <si>
+    <t>**Given** I am a banned user **when** I login, logout, view needs, search needs, and delete my account **then** the app should work fine</t>
+  </si>
+  <si>
+    <t>**Given** I am a banned user **when** I do anything else **then** the app should yell at me and not let me do that.</t>
+  </si>
+  <si>
+    <t>As a User, I want to be redirected when I am not logged in so that I can re-authenticate and continue using the website as intended.</t>
+  </si>
+  <si>
+    <t>**Given** I am logged out **when** I try to view any pages requiring an account (any page but Login and Homepage) **then** I am redirected to the login.</t>
+  </si>
+  <si>
+    <t>As a owner I want to have all tabs located in a dropdown menu so that the website looks better.</t>
+  </si>
+  <si>
+    <t>**Given** I am logged in **when** I click on the dropdown menu**then** I see the tab buttons.</t>
+  </si>
+  <si>
+    <t>As a User I want to obscure things typed into the change password/password text boxes so that people cannot see my password. (The solution will also result in the Username field changing to be the same as Password.)</t>
+  </si>
+  <si>
+    <t>**Given** that I am changing my password **when** I enter text into the change password field **then** the text that I entered is obscured.</t>
+  </si>
+  <si>
+    <t>Given that I am changing my password, when I press the change password button, then a textbox appears</t>
+  </si>
+  <si>
+    <t>Given that I am changing my password, when I press the change password button, then a confirm button appears</t>
+  </si>
+  <si>
+    <t>As a manager I want to be able to search for a user by their username so that I can refine my list of users if I am looking for someone.</t>
+  </si>
+  <si>
+    <t>**Given** I am a manager **when** I search for a username **then** I expect any user with a username that contains the text I enter to appear in the list</t>
+  </si>
+  <si>
+    <t>As a manager I want to be able to get the list of all users so that I can see who has accessed the system.</t>
+  </si>
+  <si>
+    <t>**Given** I am a manager **when** I go to the users tab **then** I expect to see a list of all the users that exist</t>
+  </si>
+  <si>
+    <t>As a Helper I want to be able to reset my password so that if I forget it I can regain access to my account.</t>
+  </si>
+  <si>
+    <t>**Given** I do not have an account **when** I create an account **then** I should be asked to make a security question</t>
+  </si>
+  <si>
+    <t>**Given** I am not logged in **when** I press the forgot password button on the login screen **then** I expect to be able to be taken to confirm I am who I say I am by answering my security question</t>
+  </si>
+  <si>
+    <t>As a Manager I want to List people who have donated recently so that people can be thanked, and people can be encouraged to donate (so that their name appears).</t>
+  </si>
+  <si>
+    <t>**Given** a user is logged in **when** I access the home page **then** I can see a more elaborate list of 'thank you's (all of the 'thank you's).</t>
+  </si>
+  <si>
+    <t>As a User I want to see the home/landing page so that I can initially access the app.</t>
+  </si>
+  <si>
+    <t>**Given** I a user is not logged in **when** they go the the site **then** they should be sent to the home page</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -265,6 +399,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -274,7 +414,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -291,11 +431,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -320,14 +469,23 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -704,34 +862,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="18.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="18.600000000000001"/>
   <cols>
     <col min="1" max="1" width="21" style="1" customWidth="1"/>
-    <col min="2" max="2" width="106.83203125" customWidth="1"/>
+    <col min="2" max="2" width="106.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="279" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="279">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -748,7 +906,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F582"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="30" style="2" customWidth="1"/>
     <col min="2" max="2" width="60" style="2" customWidth="1"/>
@@ -756,2641 +914,2893 @@
     <col min="4" max="4" width="60" style="2" customWidth="1"/>
     <col min="5" max="5" width="9" style="2" customWidth="1"/>
     <col min="6" max="6" width="60" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="10.83203125" style="5"/>
+    <col min="7" max="16384" width="10.875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" s="4" customFormat="1">
       <c r="A1" s="3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="62" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="62.1">
       <c r="A2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="7"/>
+    </row>
+    <row r="3" spans="1:6" ht="47.1" thickBot="1">
+      <c r="A3" s="11"/>
+      <c r="B3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="7"/>
+    </row>
+    <row r="4" spans="1:6" ht="47.1" thickBot="1">
+      <c r="A4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="7" t="s">
+      <c r="C4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="7"/>
+    </row>
+    <row r="5" spans="1:6" ht="62.1">
+      <c r="A5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="7"/>
+    </row>
+    <row r="6" spans="1:6" ht="31.5" thickBot="1">
+      <c r="A6" s="11"/>
+      <c r="B6" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="7"/>
+    </row>
+    <row r="7" spans="1:6" ht="47.1" thickBot="1">
+      <c r="A7" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="7"/>
+    </row>
+    <row r="8" spans="1:6" ht="62.1">
+      <c r="A8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="7"/>
+    </row>
+    <row r="9" spans="1:6" ht="31.5" thickBot="1">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="7"/>
+    </row>
+    <row r="10" spans="1:6" ht="46.5">
+      <c r="A10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="7"/>
+    </row>
+    <row r="11" spans="1:6" ht="46.5">
+      <c r="B11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="7"/>
+    </row>
+    <row r="12" spans="1:6" ht="31.5" thickBot="1">
+      <c r="A12" s="11"/>
+      <c r="B12" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="7"/>
+    </row>
+    <row r="13" spans="1:6" ht="47.1" thickBot="1">
+      <c r="A13" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="77.45">
+      <c r="A14" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="7"/>
+    </row>
+    <row r="15" spans="1:6" ht="31.5" thickBot="1">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" ht="46.5">
+      <c r="A16" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" ht="31.5" thickBot="1">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="7"/>
+    </row>
+    <row r="18" spans="1:6" ht="46.5">
+      <c r="A18" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" ht="46.5">
+      <c r="B19" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" ht="31.5" thickBot="1">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="7"/>
+    </row>
+    <row r="21" spans="1:6" ht="46.5">
+      <c r="A21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="7"/>
+    </row>
+    <row r="22" spans="1:6" ht="30.95">
+      <c r="B22" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="7"/>
+    </row>
+    <row r="23" spans="1:6" ht="31.5" thickBot="1">
+      <c r="A23" s="11"/>
+      <c r="B23" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" s="7"/>
+    </row>
+    <row r="24" spans="1:6" ht="46.5">
+      <c r="A24" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="7"/>
+    </row>
+    <row r="25" spans="1:6" ht="31.5" thickBot="1">
+      <c r="A25" s="11"/>
+      <c r="B25" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="7"/>
+    </row>
+    <row r="26" spans="1:6" ht="46.5">
+      <c r="A26" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="C26" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="7"/>
+    </row>
+    <row r="27" spans="1:6" ht="31.5" thickBot="1">
+      <c r="A27" s="11"/>
+      <c r="B27" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="7"/>
-    </row>
-    <row r="3" spans="1:6" ht="47" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E3" s="7"/>
-    </row>
-    <row r="4" spans="1:6" ht="47" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" s="7"/>
-    </row>
-    <row r="5" spans="1:6" ht="62" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E5" s="7"/>
-    </row>
-    <row r="6" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12" t="s">
+      <c r="C27" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" s="7"/>
+    </row>
+    <row r="28" spans="1:6" ht="48.75">
+      <c r="A28" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="48.75">
+      <c r="A29" s="13"/>
+      <c r="B29" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="64.5">
+      <c r="A30" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E6" s="7"/>
-    </row>
-    <row r="7" spans="1:6" ht="47" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E7" s="7"/>
-    </row>
-    <row r="8" spans="1:6" ht="62" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E8" s="7"/>
-    </row>
-    <row r="9" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" s="7"/>
-    </row>
-    <row r="10" spans="1:6" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" s="7"/>
-    </row>
-    <row r="11" spans="1:6" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="B11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E11" s="7"/>
-    </row>
-    <row r="12" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E12" s="7"/>
-    </row>
-    <row r="13" spans="1:6" ht="47" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" s="7"/>
-    </row>
-    <row r="14" spans="1:6" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="E14" s="7"/>
-    </row>
-    <row r="15" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="7"/>
-    </row>
-    <row r="16" spans="1:6" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E16" s="7"/>
-    </row>
-    <row r="17" spans="1:5" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E17" s="7"/>
-    </row>
-    <row r="18" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E18" s="7"/>
-    </row>
-    <row r="19" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="B19" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" s="7"/>
-    </row>
-    <row r="20" spans="1:5" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E20" s="7"/>
-    </row>
-    <row r="21" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E21" s="7"/>
-    </row>
-    <row r="22" spans="1:5" ht="31" x14ac:dyDescent="0.35">
-      <c r="B22" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E22" s="7"/>
-    </row>
-    <row r="23" spans="1:5" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="7"/>
-    </row>
-    <row r="24" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E24" s="7"/>
-    </row>
-    <row r="25" spans="1:5" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E25" s="7"/>
-    </row>
-    <row r="26" spans="1:5" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E26" s="7"/>
-    </row>
-    <row r="27" spans="1:5" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D27" s="2" t="s">
+      <c r="E30" s="7"/>
+    </row>
+    <row r="31" spans="1:6" ht="81">
+      <c r="A31" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" s="7"/>
+      <c r="E31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E27" s="7"/>
-    </row>
-    <row r="28" spans="1:5" ht="62" x14ac:dyDescent="0.35">
-      <c r="A28" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E28" s="7"/>
-    </row>
-    <row r="29" spans="1:5" ht="47" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E29" s="7"/>
-    </row>
-    <row r="30" spans="1:5" ht="62" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E30" s="7"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C31" s="7"/>
-      <c r="E31" s="7"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="6"/>
+    </row>
+    <row r="32" spans="1:6" ht="48.75">
+      <c r="A32" s="14"/>
+      <c r="B32" s="13" t="s">
+        <v>67</v>
+      </c>
       <c r="C32" s="7"/>
-      <c r="E32" s="7"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="6"/>
+      <c r="E32" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="48.75">
+      <c r="A33" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="C33" s="7"/>
-      <c r="E33" s="7"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E33" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="32.25">
+      <c r="A34" s="13"/>
+      <c r="B34" s="13" t="s">
+        <v>70</v>
+      </c>
       <c r="C34" s="7"/>
-      <c r="E34" s="7"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="6"/>
+      <c r="E34" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="48.75">
+      <c r="A35" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>72</v>
+      </c>
       <c r="C35" s="7"/>
-      <c r="E35" s="7"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E35" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="32.25">
+      <c r="A36" s="13"/>
+      <c r="B36" s="13" t="s">
+        <v>73</v>
+      </c>
       <c r="C36" s="7"/>
-      <c r="E36" s="7"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E36" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="48.75">
+      <c r="A37" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>75</v>
+      </c>
       <c r="C37" s="7"/>
-      <c r="E37" s="7"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E37" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="32.25">
+      <c r="A38" s="13"/>
+      <c r="B38" s="13" t="s">
+        <v>76</v>
+      </c>
       <c r="C38" s="7"/>
-      <c r="E38" s="7"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E38" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="48.75">
+      <c r="A39" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>78</v>
+      </c>
       <c r="C39" s="7"/>
-      <c r="E39" s="7"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E39" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="64.5">
+      <c r="A40" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>80</v>
+      </c>
       <c r="C40" s="7"/>
-      <c r="E40" s="7"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E40" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="48.75">
+      <c r="A41" s="13"/>
+      <c r="B41" s="13" t="s">
+        <v>81</v>
+      </c>
       <c r="C41" s="7"/>
-      <c r="E41" s="7"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E41" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="96.75">
+      <c r="A42" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="C42" s="7"/>
-      <c r="E42" s="7"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E42" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="32.25">
+      <c r="A43" s="13"/>
+      <c r="B43" s="13" t="s">
+        <v>84</v>
+      </c>
       <c r="C43" s="7"/>
-      <c r="E43" s="7"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E43" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="64.5">
+      <c r="A44" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B44" s="13" t="s">
+        <v>86</v>
+      </c>
       <c r="C44" s="7"/>
-      <c r="E44" s="7"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E44" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="48.75">
+      <c r="A45" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>88</v>
+      </c>
       <c r="C45" s="7"/>
-      <c r="E45" s="7"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E45" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="113.25">
+      <c r="A46" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="C46" s="7"/>
-      <c r="E46" s="7"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E46" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="32.25">
+      <c r="B47" s="2" t="s">
+        <v>91</v>
+      </c>
       <c r="C47" s="7"/>
-      <c r="E47" s="7"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E47" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="32.25">
+      <c r="A48" s="13"/>
+      <c r="B48" s="13" t="s">
+        <v>92</v>
+      </c>
       <c r="C48" s="7"/>
-      <c r="E48" s="7"/>
-    </row>
-    <row r="49" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E48" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="64.5">
+      <c r="A49" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B49" s="13" t="s">
+        <v>94</v>
+      </c>
       <c r="C49" s="7"/>
-      <c r="E49" s="7"/>
-    </row>
-    <row r="50" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E49" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="48.75">
+      <c r="A50" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B50" s="13" t="s">
+        <v>96</v>
+      </c>
       <c r="C50" s="7"/>
-      <c r="E50" s="7"/>
-    </row>
-    <row r="51" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E50" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="48.75">
+      <c r="A51" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>98</v>
+      </c>
       <c r="C51" s="7"/>
-      <c r="E51" s="7"/>
-    </row>
-    <row r="52" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E51" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="48.75">
+      <c r="A52" s="13"/>
+      <c r="B52" s="13" t="s">
+        <v>99</v>
+      </c>
       <c r="C52" s="7"/>
-      <c r="E52" s="7"/>
-    </row>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E52" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="81">
+      <c r="A53" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>101</v>
+      </c>
       <c r="C53" s="7"/>
-      <c r="E53" s="7"/>
-    </row>
-    <row r="54" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E53" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="48.75">
+      <c r="A54" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>103</v>
+      </c>
       <c r="C54" s="7"/>
-      <c r="E54" s="7"/>
-    </row>
-    <row r="55" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E54" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="15.75">
       <c r="C55" s="7"/>
       <c r="E55" s="7"/>
     </row>
-    <row r="56" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" ht="15.75">
       <c r="C56" s="7"/>
       <c r="E56" s="7"/>
     </row>
-    <row r="57" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6">
       <c r="C57" s="7"/>
       <c r="E57" s="7"/>
     </row>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6">
       <c r="C58" s="7"/>
       <c r="E58" s="7"/>
     </row>
-    <row r="59" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6">
       <c r="C59" s="7"/>
       <c r="E59" s="7"/>
     </row>
-    <row r="60" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6">
       <c r="C60" s="7"/>
       <c r="E60" s="7"/>
     </row>
-    <row r="61" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6">
       <c r="C61" s="7"/>
       <c r="E61" s="7"/>
     </row>
-    <row r="62" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6">
       <c r="C62" s="7"/>
       <c r="E62" s="7"/>
     </row>
-    <row r="63" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6">
       <c r="C63" s="7"/>
       <c r="E63" s="7"/>
     </row>
-    <row r="64" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6">
       <c r="C64" s="7"/>
       <c r="E64" s="7"/>
     </row>
-    <row r="65" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="3:5">
       <c r="C65" s="7"/>
       <c r="E65" s="7"/>
     </row>
-    <row r="66" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="3:5">
       <c r="C66" s="7"/>
       <c r="E66" s="7"/>
     </row>
-    <row r="67" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="3:5">
       <c r="C67" s="7"/>
       <c r="E67" s="7"/>
     </row>
-    <row r="68" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="3:5">
       <c r="C68" s="7"/>
       <c r="E68" s="7"/>
     </row>
-    <row r="69" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="3:5">
       <c r="C69" s="7"/>
       <c r="E69" s="7"/>
     </row>
-    <row r="70" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="3:5">
       <c r="C70" s="7"/>
       <c r="E70" s="7"/>
     </row>
-    <row r="71" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="3:5">
       <c r="C71" s="7"/>
       <c r="E71" s="7"/>
     </row>
-    <row r="72" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="3:5">
       <c r="C72" s="7"/>
       <c r="E72" s="7"/>
     </row>
-    <row r="73" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="3:5">
       <c r="C73" s="7"/>
       <c r="E73" s="7"/>
     </row>
-    <row r="74" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="3:5">
       <c r="C74" s="7"/>
       <c r="E74" s="7"/>
     </row>
-    <row r="75" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="3:5">
       <c r="C75" s="7"/>
       <c r="E75" s="7"/>
     </row>
-    <row r="76" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="3:5">
       <c r="C76" s="7"/>
       <c r="E76" s="7"/>
     </row>
-    <row r="77" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="3:5">
       <c r="C77" s="7"/>
       <c r="E77" s="7"/>
     </row>
-    <row r="78" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="3:5">
       <c r="C78" s="7"/>
       <c r="E78" s="7"/>
     </row>
-    <row r="79" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="3:5">
       <c r="C79" s="7"/>
       <c r="E79" s="7"/>
     </row>
-    <row r="80" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="3:5">
       <c r="C80" s="7"/>
       <c r="E80" s="7"/>
     </row>
-    <row r="81" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="3:5">
       <c r="C81" s="7"/>
       <c r="E81" s="7"/>
     </row>
-    <row r="82" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="3:5">
       <c r="C82" s="7"/>
       <c r="E82" s="7"/>
     </row>
-    <row r="83" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="3:5">
       <c r="C83" s="7"/>
       <c r="E83" s="7"/>
     </row>
-    <row r="84" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="3:5">
       <c r="C84" s="7"/>
       <c r="E84" s="7"/>
     </row>
-    <row r="85" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="3:5">
       <c r="C85" s="7"/>
       <c r="E85" s="7"/>
     </row>
-    <row r="86" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="3:5">
       <c r="C86" s="7"/>
       <c r="E86" s="7"/>
     </row>
-    <row r="87" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="3:5">
       <c r="C87" s="7"/>
       <c r="E87" s="7"/>
     </row>
-    <row r="88" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="3:5">
       <c r="C88" s="7"/>
       <c r="E88" s="7"/>
     </row>
-    <row r="89" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="3:5">
       <c r="C89" s="7"/>
       <c r="E89" s="7"/>
     </row>
-    <row r="90" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="3:5">
       <c r="C90" s="7"/>
       <c r="E90" s="7"/>
     </row>
-    <row r="91" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="3:5">
       <c r="C91" s="7"/>
       <c r="E91" s="7"/>
     </row>
-    <row r="92" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="3:5">
       <c r="C92" s="7"/>
       <c r="E92" s="7"/>
     </row>
-    <row r="93" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="3:5">
       <c r="C93" s="7"/>
       <c r="E93" s="7"/>
     </row>
-    <row r="94" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="3:5">
       <c r="C94" s="7"/>
       <c r="E94" s="7"/>
     </row>
-    <row r="95" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="3:5">
       <c r="C95" s="7"/>
       <c r="E95" s="7"/>
     </row>
-    <row r="96" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="3:5">
       <c r="C96" s="7"/>
       <c r="E96" s="7"/>
     </row>
-    <row r="97" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="3:5">
       <c r="C97" s="7"/>
       <c r="E97" s="7"/>
     </row>
-    <row r="98" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="3:5">
       <c r="C98" s="7"/>
       <c r="E98" s="7"/>
     </row>
-    <row r="99" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="3:5">
       <c r="C99" s="7"/>
       <c r="E99" s="7"/>
     </row>
-    <row r="100" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="3:5">
       <c r="C100" s="7"/>
       <c r="E100" s="7"/>
     </row>
-    <row r="101" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="3:5">
       <c r="C101" s="7"/>
       <c r="E101" s="7"/>
     </row>
-    <row r="102" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="3:5">
       <c r="C102" s="7"/>
       <c r="E102" s="7"/>
     </row>
-    <row r="103" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="3:5">
       <c r="C103" s="7"/>
       <c r="E103" s="7"/>
     </row>
-    <row r="104" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="3:5">
       <c r="C104" s="7"/>
       <c r="E104" s="7"/>
     </row>
-    <row r="105" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="3:5">
       <c r="C105" s="7"/>
       <c r="E105" s="7"/>
     </row>
-    <row r="106" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="3:5">
       <c r="C106" s="7"/>
       <c r="E106" s="7"/>
     </row>
-    <row r="107" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="3:5">
       <c r="C107" s="7"/>
       <c r="E107" s="7"/>
     </row>
-    <row r="108" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="3:5">
       <c r="C108" s="7"/>
       <c r="E108" s="7"/>
     </row>
-    <row r="109" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="3:5">
       <c r="C109" s="7"/>
       <c r="E109" s="7"/>
     </row>
-    <row r="110" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="3:5">
       <c r="C110" s="7"/>
       <c r="E110" s="7"/>
     </row>
-    <row r="111" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="3:5">
       <c r="C111" s="7"/>
       <c r="E111" s="7"/>
     </row>
-    <row r="112" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="3:5">
       <c r="C112" s="7"/>
       <c r="E112" s="7"/>
     </row>
-    <row r="113" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="3:5">
       <c r="C113" s="7"/>
       <c r="E113" s="7"/>
     </row>
-    <row r="114" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="3:5">
       <c r="C114" s="7"/>
       <c r="E114" s="7"/>
     </row>
-    <row r="115" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="3:5">
       <c r="C115" s="7"/>
       <c r="E115" s="7"/>
     </row>
-    <row r="116" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="3:5">
       <c r="C116" s="7"/>
       <c r="E116" s="7"/>
     </row>
-    <row r="117" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="3:5">
       <c r="C117" s="7"/>
       <c r="E117" s="7"/>
     </row>
-    <row r="118" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="3:5">
       <c r="C118" s="7"/>
       <c r="E118" s="7"/>
     </row>
-    <row r="119" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="3:5">
       <c r="C119" s="7"/>
       <c r="E119" s="7"/>
     </row>
-    <row r="120" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="3:5">
       <c r="C120" s="7"/>
       <c r="E120" s="7"/>
     </row>
-    <row r="121" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="3:5">
       <c r="C121" s="7"/>
       <c r="E121" s="7"/>
     </row>
-    <row r="122" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="3:5">
       <c r="C122" s="7"/>
       <c r="E122" s="7"/>
     </row>
-    <row r="123" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="3:5">
       <c r="C123" s="7"/>
       <c r="E123" s="7"/>
     </row>
-    <row r="124" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="3:5">
       <c r="C124" s="7"/>
       <c r="E124" s="7"/>
     </row>
-    <row r="125" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="3:5">
       <c r="C125" s="7"/>
       <c r="E125" s="7"/>
     </row>
-    <row r="126" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="3:5">
       <c r="C126" s="7"/>
       <c r="E126" s="7"/>
     </row>
-    <row r="127" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="3:5">
       <c r="C127" s="7"/>
       <c r="E127" s="7"/>
     </row>
-    <row r="128" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="3:5">
       <c r="C128" s="7"/>
       <c r="E128" s="7"/>
     </row>
-    <row r="129" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="3:5">
       <c r="C129" s="7"/>
       <c r="E129" s="7"/>
     </row>
-    <row r="130" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="3:5">
       <c r="C130" s="7"/>
       <c r="E130" s="7"/>
     </row>
-    <row r="131" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="3:5">
       <c r="C131" s="7"/>
       <c r="E131" s="7"/>
     </row>
-    <row r="132" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="3:5">
       <c r="C132" s="7"/>
       <c r="E132" s="7"/>
     </row>
-    <row r="133" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="3:5">
       <c r="C133" s="7"/>
       <c r="E133" s="7"/>
     </row>
-    <row r="134" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="3:5">
       <c r="C134" s="7"/>
       <c r="E134" s="7"/>
     </row>
-    <row r="135" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="3:5">
       <c r="C135" s="7"/>
       <c r="E135" s="7"/>
     </row>
-    <row r="136" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="3:5">
       <c r="C136" s="7"/>
       <c r="E136" s="7"/>
     </row>
-    <row r="137" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="3:5">
       <c r="C137" s="7"/>
       <c r="E137" s="7"/>
     </row>
-    <row r="138" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="3:5">
       <c r="C138" s="7"/>
       <c r="E138" s="7"/>
     </row>
-    <row r="139" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="3:5">
       <c r="C139" s="7"/>
       <c r="E139" s="7"/>
     </row>
-    <row r="140" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="3:5">
       <c r="C140" s="7"/>
       <c r="E140" s="7"/>
     </row>
-    <row r="141" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="3:5">
       <c r="C141" s="7"/>
       <c r="E141" s="7"/>
     </row>
-    <row r="142" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="3:5">
       <c r="C142" s="7"/>
       <c r="E142" s="7"/>
     </row>
-    <row r="143" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="3:5">
       <c r="C143" s="7"/>
       <c r="E143" s="7"/>
     </row>
-    <row r="144" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="3:5">
       <c r="C144" s="7"/>
       <c r="E144" s="7"/>
     </row>
-    <row r="145" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="3:5">
       <c r="C145" s="7"/>
       <c r="E145" s="7"/>
     </row>
-    <row r="146" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="3:5">
       <c r="C146" s="7"/>
       <c r="E146" s="7"/>
     </row>
-    <row r="147" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="3:5">
       <c r="C147" s="7"/>
       <c r="E147" s="7"/>
     </row>
-    <row r="148" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="3:5">
       <c r="C148" s="7"/>
       <c r="E148" s="7"/>
     </row>
-    <row r="149" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="3:5">
       <c r="C149" s="7"/>
       <c r="E149" s="7"/>
     </row>
-    <row r="150" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="3:5">
       <c r="C150" s="7"/>
       <c r="E150" s="7"/>
     </row>
-    <row r="151" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="3:5">
       <c r="C151" s="7"/>
       <c r="E151" s="7"/>
     </row>
-    <row r="152" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="3:5">
       <c r="C152" s="7"/>
       <c r="E152" s="7"/>
     </row>
-    <row r="153" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="3:5">
       <c r="C153" s="7"/>
       <c r="E153" s="7"/>
     </row>
-    <row r="154" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="3:5">
       <c r="C154" s="7"/>
       <c r="E154" s="7"/>
     </row>
-    <row r="155" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="3:5">
       <c r="C155" s="7"/>
       <c r="E155" s="7"/>
     </row>
-    <row r="156" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="3:5">
       <c r="C156" s="7"/>
       <c r="E156" s="7"/>
     </row>
-    <row r="157" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="3:5">
       <c r="C157" s="7"/>
       <c r="E157" s="7"/>
     </row>
-    <row r="158" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="3:5">
       <c r="C158" s="7"/>
       <c r="E158" s="7"/>
     </row>
-    <row r="159" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="3:5">
       <c r="C159" s="7"/>
       <c r="E159" s="7"/>
     </row>
-    <row r="160" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="3:5">
       <c r="C160" s="7"/>
       <c r="E160" s="7"/>
     </row>
-    <row r="161" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="3:5">
       <c r="C161" s="7"/>
       <c r="E161" s="7"/>
     </row>
-    <row r="162" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="3:5">
       <c r="C162" s="7"/>
       <c r="E162" s="7"/>
     </row>
-    <row r="163" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="3:5">
       <c r="C163" s="7"/>
       <c r="E163" s="7"/>
     </row>
-    <row r="164" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="3:5">
       <c r="C164" s="7"/>
       <c r="E164" s="7"/>
     </row>
-    <row r="165" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="3:5">
       <c r="C165" s="7"/>
       <c r="E165" s="7"/>
     </row>
-    <row r="166" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="3:5">
       <c r="C166" s="7"/>
       <c r="E166" s="7"/>
     </row>
-    <row r="167" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="3:5">
       <c r="C167" s="7"/>
       <c r="E167" s="7"/>
     </row>
-    <row r="168" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="3:5">
       <c r="C168" s="7"/>
       <c r="E168" s="7"/>
     </row>
-    <row r="169" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="3:5">
       <c r="C169" s="7"/>
       <c r="E169" s="7"/>
     </row>
-    <row r="170" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="3:5">
       <c r="C170" s="7"/>
       <c r="E170" s="7"/>
     </row>
-    <row r="171" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="3:5">
       <c r="C171" s="7"/>
       <c r="E171" s="7"/>
     </row>
-    <row r="172" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="3:5">
       <c r="C172" s="7"/>
       <c r="E172" s="7"/>
     </row>
-    <row r="173" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="3:5">
       <c r="C173" s="7"/>
       <c r="E173" s="7"/>
     </row>
-    <row r="174" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="3:5">
       <c r="C174" s="7"/>
       <c r="E174" s="7"/>
     </row>
-    <row r="175" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="3:5">
       <c r="C175" s="7"/>
       <c r="E175" s="7"/>
     </row>
-    <row r="176" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="3:5">
       <c r="C176" s="7"/>
       <c r="E176" s="7"/>
     </row>
-    <row r="177" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="3:5">
       <c r="C177" s="7"/>
       <c r="E177" s="7"/>
     </row>
-    <row r="178" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="3:5">
       <c r="C178" s="7"/>
       <c r="E178" s="7"/>
     </row>
-    <row r="179" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="3:5">
       <c r="C179" s="7"/>
       <c r="E179" s="7"/>
     </row>
-    <row r="180" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="3:5">
       <c r="C180" s="7"/>
       <c r="E180" s="7"/>
     </row>
-    <row r="181" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="3:5">
       <c r="C181" s="7"/>
       <c r="E181" s="7"/>
     </row>
-    <row r="182" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="3:5">
       <c r="C182" s="7"/>
       <c r="E182" s="7"/>
     </row>
-    <row r="183" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="3:5">
       <c r="C183" s="7"/>
       <c r="E183" s="7"/>
     </row>
-    <row r="184" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="3:5">
       <c r="C184" s="7"/>
       <c r="E184" s="7"/>
     </row>
-    <row r="185" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="3:5">
       <c r="C185" s="7"/>
       <c r="E185" s="7"/>
     </row>
-    <row r="186" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="3:5">
       <c r="C186" s="7"/>
       <c r="E186" s="7"/>
     </row>
-    <row r="187" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="3:5">
       <c r="C187" s="7"/>
       <c r="E187" s="7"/>
     </row>
-    <row r="188" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="3:5">
       <c r="C188" s="7"/>
       <c r="E188" s="7"/>
     </row>
-    <row r="189" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="3:5">
       <c r="C189" s="7"/>
       <c r="E189" s="7"/>
     </row>
-    <row r="190" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="3:5">
       <c r="C190" s="7"/>
       <c r="E190" s="7"/>
     </row>
-    <row r="191" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="3:5">
       <c r="C191" s="7"/>
       <c r="E191" s="7"/>
     </row>
-    <row r="192" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="3:5">
       <c r="C192" s="7"/>
       <c r="E192" s="7"/>
     </row>
-    <row r="193" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="3:5">
       <c r="C193" s="7"/>
       <c r="E193" s="7"/>
     </row>
-    <row r="194" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="3:5">
       <c r="C194" s="7"/>
       <c r="E194" s="7"/>
     </row>
-    <row r="195" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="3:5">
       <c r="C195" s="7"/>
       <c r="E195" s="7"/>
     </row>
-    <row r="196" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="3:5">
       <c r="C196" s="7"/>
       <c r="E196" s="7"/>
     </row>
-    <row r="197" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="3:5">
       <c r="C197" s="7"/>
       <c r="E197" s="7"/>
     </row>
-    <row r="198" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="3:5">
       <c r="C198" s="7"/>
       <c r="E198" s="7"/>
     </row>
-    <row r="199" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="3:5">
       <c r="C199" s="7"/>
       <c r="E199" s="7"/>
     </row>
-    <row r="200" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="3:5">
       <c r="C200" s="7"/>
       <c r="E200" s="7"/>
     </row>
-    <row r="201" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="3:5">
       <c r="C201" s="7"/>
       <c r="E201" s="7"/>
     </row>
-    <row r="202" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="3:5">
       <c r="C202" s="7"/>
       <c r="E202" s="7"/>
     </row>
-    <row r="203" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="3:5">
       <c r="C203" s="7"/>
       <c r="E203" s="7"/>
     </row>
-    <row r="204" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="3:5">
       <c r="C204" s="7"/>
       <c r="E204" s="7"/>
     </row>
-    <row r="205" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="3:5">
       <c r="C205" s="7"/>
       <c r="E205" s="7"/>
     </row>
-    <row r="206" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="3:5">
       <c r="C206" s="7"/>
       <c r="E206" s="7"/>
     </row>
-    <row r="207" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="3:5">
       <c r="C207" s="7"/>
       <c r="E207" s="7"/>
     </row>
-    <row r="208" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="3:5">
       <c r="C208" s="7"/>
       <c r="E208" s="7"/>
     </row>
-    <row r="209" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="3:5">
       <c r="C209" s="7"/>
       <c r="E209" s="7"/>
     </row>
-    <row r="210" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="3:5">
       <c r="C210" s="7"/>
       <c r="E210" s="7"/>
     </row>
-    <row r="211" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="3:5">
       <c r="C211" s="7"/>
       <c r="E211" s="7"/>
     </row>
-    <row r="212" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="3:5">
       <c r="C212" s="7"/>
       <c r="E212" s="7"/>
     </row>
-    <row r="213" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="3:5">
       <c r="C213" s="7"/>
       <c r="E213" s="7"/>
     </row>
-    <row r="214" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="3:5">
       <c r="C214" s="7"/>
       <c r="E214" s="7"/>
     </row>
-    <row r="215" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="3:5">
       <c r="C215" s="7"/>
       <c r="E215" s="7"/>
     </row>
-    <row r="216" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="3:5">
       <c r="C216" s="7"/>
       <c r="E216" s="7"/>
     </row>
-    <row r="217" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="3:5">
       <c r="C217" s="7"/>
       <c r="E217" s="7"/>
     </row>
-    <row r="218" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="3:5">
       <c r="C218" s="7"/>
       <c r="E218" s="7"/>
     </row>
-    <row r="219" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="3:5">
       <c r="C219" s="7"/>
       <c r="E219" s="7"/>
     </row>
-    <row r="220" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="3:5">
       <c r="C220" s="7"/>
       <c r="E220" s="7"/>
     </row>
-    <row r="221" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="3:5">
       <c r="C221" s="7"/>
       <c r="E221" s="7"/>
     </row>
-    <row r="222" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="3:5">
       <c r="C222" s="7"/>
       <c r="E222" s="7"/>
     </row>
-    <row r="223" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="3:5">
       <c r="C223" s="7"/>
       <c r="E223" s="7"/>
     </row>
-    <row r="224" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="3:5">
       <c r="C224" s="7"/>
       <c r="E224" s="7"/>
     </row>
-    <row r="225" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="3:5">
       <c r="C225" s="7"/>
       <c r="E225" s="7"/>
     </row>
-    <row r="226" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="3:5">
       <c r="C226" s="7"/>
       <c r="E226" s="7"/>
     </row>
-    <row r="227" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="3:5">
       <c r="C227" s="7"/>
       <c r="E227" s="7"/>
     </row>
-    <row r="228" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="3:5">
       <c r="C228" s="7"/>
       <c r="E228" s="7"/>
     </row>
-    <row r="229" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="3:5">
       <c r="C229" s="7"/>
       <c r="E229" s="7"/>
     </row>
-    <row r="230" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="3:5">
       <c r="C230" s="7"/>
       <c r="E230" s="7"/>
     </row>
-    <row r="231" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="3:5">
       <c r="C231" s="7"/>
       <c r="E231" s="7"/>
     </row>
-    <row r="232" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="3:5">
       <c r="C232" s="7"/>
       <c r="E232" s="7"/>
     </row>
-    <row r="233" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="3:5">
       <c r="C233" s="7"/>
       <c r="E233" s="7"/>
     </row>
-    <row r="234" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="3:5">
       <c r="C234" s="7"/>
       <c r="E234" s="7"/>
     </row>
-    <row r="235" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="3:5">
       <c r="C235" s="7"/>
       <c r="E235" s="7"/>
     </row>
-    <row r="236" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="3:5">
       <c r="C236" s="7"/>
       <c r="E236" s="7"/>
     </row>
-    <row r="237" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="3:5">
       <c r="C237" s="7"/>
       <c r="E237" s="7"/>
     </row>
-    <row r="238" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="3:5">
       <c r="C238" s="7"/>
       <c r="E238" s="7"/>
     </row>
-    <row r="239" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="3:5">
       <c r="C239" s="7"/>
       <c r="E239" s="7"/>
     </row>
-    <row r="240" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="3:5">
       <c r="C240" s="7"/>
       <c r="E240" s="7"/>
     </row>
-    <row r="241" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="3:5">
       <c r="C241" s="7"/>
       <c r="E241" s="7"/>
     </row>
-    <row r="242" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="3:5">
       <c r="C242" s="7"/>
       <c r="E242" s="7"/>
     </row>
-    <row r="243" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="3:5">
       <c r="C243" s="7"/>
       <c r="E243" s="7"/>
     </row>
-    <row r="244" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="3:5">
       <c r="C244" s="7"/>
       <c r="E244" s="7"/>
     </row>
-    <row r="245" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="3:5">
       <c r="C245" s="7"/>
       <c r="E245" s="7"/>
     </row>
-    <row r="246" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="3:5">
       <c r="C246" s="7"/>
       <c r="E246" s="7"/>
     </row>
-    <row r="247" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="3:5">
       <c r="C247" s="7"/>
       <c r="E247" s="7"/>
     </row>
-    <row r="248" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="3:5">
       <c r="C248" s="7"/>
       <c r="E248" s="7"/>
     </row>
-    <row r="249" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="3:5">
       <c r="C249" s="7"/>
       <c r="E249" s="7"/>
     </row>
-    <row r="250" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="3:5">
       <c r="C250" s="7"/>
       <c r="E250" s="7"/>
     </row>
-    <row r="251" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="3:5">
       <c r="C251" s="7"/>
       <c r="E251" s="7"/>
     </row>
-    <row r="252" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="3:5">
       <c r="C252" s="7"/>
       <c r="E252" s="7"/>
     </row>
-    <row r="253" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="3:5">
       <c r="C253" s="7"/>
       <c r="E253" s="7"/>
     </row>
-    <row r="254" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="3:5">
       <c r="C254" s="7"/>
       <c r="E254" s="7"/>
     </row>
-    <row r="255" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="3:5">
       <c r="C255" s="7"/>
       <c r="E255" s="7"/>
     </row>
-    <row r="256" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="3:5">
       <c r="C256" s="7"/>
       <c r="E256" s="7"/>
     </row>
-    <row r="257" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="3:5">
       <c r="C257" s="7"/>
       <c r="E257" s="7"/>
     </row>
-    <row r="258" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="3:5">
       <c r="C258" s="7"/>
       <c r="E258" s="7"/>
     </row>
-    <row r="259" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="3:5">
       <c r="C259" s="7"/>
       <c r="E259" s="7"/>
     </row>
-    <row r="260" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="3:5">
       <c r="C260" s="7"/>
       <c r="E260" s="7"/>
     </row>
-    <row r="261" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="3:5">
       <c r="C261" s="7"/>
       <c r="E261" s="7"/>
     </row>
-    <row r="262" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="3:5">
       <c r="C262" s="7"/>
       <c r="E262" s="7"/>
     </row>
-    <row r="263" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="3:5">
       <c r="C263" s="7"/>
       <c r="E263" s="7"/>
     </row>
-    <row r="264" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="3:5">
       <c r="C264" s="7"/>
       <c r="E264" s="7"/>
     </row>
-    <row r="265" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="3:5">
       <c r="C265" s="7"/>
       <c r="E265" s="7"/>
     </row>
-    <row r="266" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="3:5">
       <c r="C266" s="7"/>
       <c r="E266" s="7"/>
     </row>
-    <row r="267" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="3:5">
       <c r="C267" s="7"/>
       <c r="E267" s="7"/>
     </row>
-    <row r="268" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="3:5">
       <c r="C268" s="7"/>
       <c r="E268" s="7"/>
     </row>
-    <row r="269" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="3:5">
       <c r="C269" s="7"/>
       <c r="E269" s="7"/>
     </row>
-    <row r="270" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="3:5">
       <c r="C270" s="7"/>
       <c r="E270" s="7"/>
     </row>
-    <row r="271" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="3:5">
       <c r="C271" s="7"/>
       <c r="E271" s="7"/>
     </row>
-    <row r="272" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="3:5">
       <c r="C272" s="7"/>
       <c r="E272" s="7"/>
     </row>
-    <row r="273" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="3:5">
       <c r="C273" s="7"/>
       <c r="E273" s="7"/>
     </row>
-    <row r="274" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="3:5">
       <c r="C274" s="7"/>
       <c r="E274" s="7"/>
     </row>
-    <row r="275" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="3:5">
       <c r="C275" s="7"/>
       <c r="E275" s="7"/>
     </row>
-    <row r="276" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="3:5">
       <c r="C276" s="7"/>
       <c r="E276" s="7"/>
     </row>
-    <row r="277" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="3:5">
       <c r="C277" s="7"/>
       <c r="E277" s="7"/>
     </row>
-    <row r="278" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="3:5">
       <c r="C278" s="7"/>
       <c r="E278" s="7"/>
     </row>
-    <row r="279" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="3:5">
       <c r="C279" s="7"/>
       <c r="E279" s="7"/>
     </row>
-    <row r="280" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="3:5">
       <c r="C280" s="7"/>
       <c r="E280" s="7"/>
     </row>
-    <row r="281" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="3:5">
       <c r="C281" s="7"/>
       <c r="E281" s="7"/>
     </row>
-    <row r="282" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="3:5">
       <c r="C282" s="7"/>
       <c r="E282" s="7"/>
     </row>
-    <row r="283" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="3:5">
       <c r="C283" s="7"/>
       <c r="E283" s="7"/>
     </row>
-    <row r="284" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="3:5">
       <c r="C284" s="7"/>
       <c r="E284" s="7"/>
     </row>
-    <row r="285" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="3:5">
       <c r="C285" s="7"/>
       <c r="E285" s="7"/>
     </row>
-    <row r="286" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="3:5">
       <c r="C286" s="7"/>
       <c r="E286" s="7"/>
     </row>
-    <row r="287" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="3:5">
       <c r="C287" s="7"/>
       <c r="E287" s="7"/>
     </row>
-    <row r="288" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="3:5">
       <c r="C288" s="7"/>
       <c r="E288" s="7"/>
     </row>
-    <row r="289" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="3:5">
       <c r="C289" s="7"/>
       <c r="E289" s="7"/>
     </row>
-    <row r="290" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="3:5">
       <c r="C290" s="7"/>
       <c r="E290" s="7"/>
     </row>
-    <row r="291" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="3:5">
       <c r="C291" s="7"/>
       <c r="E291" s="7"/>
     </row>
-    <row r="292" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="3:5">
       <c r="C292" s="7"/>
       <c r="E292" s="7"/>
     </row>
-    <row r="293" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="3:5">
       <c r="C293" s="7"/>
       <c r="E293" s="7"/>
     </row>
-    <row r="294" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="3:5">
       <c r="C294" s="7"/>
       <c r="E294" s="7"/>
     </row>
-    <row r="295" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="3:5">
       <c r="C295" s="7"/>
       <c r="E295" s="7"/>
     </row>
-    <row r="296" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="3:5">
       <c r="C296" s="7"/>
       <c r="E296" s="7"/>
     </row>
-    <row r="297" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="3:5">
       <c r="C297" s="7"/>
       <c r="E297" s="7"/>
     </row>
-    <row r="298" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="3:5">
       <c r="C298" s="7"/>
       <c r="E298" s="7"/>
     </row>
-    <row r="299" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="3:5">
       <c r="C299" s="7"/>
       <c r="E299" s="7"/>
     </row>
-    <row r="300" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="3:5">
       <c r="C300" s="7"/>
       <c r="E300" s="7"/>
     </row>
-    <row r="301" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="3:5">
       <c r="C301" s="7"/>
       <c r="E301" s="7"/>
     </row>
-    <row r="302" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="3:5">
       <c r="C302" s="7"/>
       <c r="E302" s="7"/>
     </row>
-    <row r="303" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="3:5">
       <c r="C303" s="7"/>
       <c r="E303" s="7"/>
     </row>
-    <row r="304" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="3:5">
       <c r="C304" s="7"/>
       <c r="E304" s="7"/>
     </row>
-    <row r="305" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="3:5">
       <c r="C305" s="7"/>
       <c r="E305" s="7"/>
     </row>
-    <row r="306" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="3:5">
       <c r="C306" s="7"/>
       <c r="E306" s="7"/>
     </row>
-    <row r="307" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="3:5">
       <c r="C307" s="7"/>
       <c r="E307" s="7"/>
     </row>
-    <row r="308" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="3:5">
       <c r="C308" s="7"/>
       <c r="E308" s="7"/>
     </row>
-    <row r="309" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="3:5">
       <c r="C309" s="7"/>
       <c r="E309" s="7"/>
     </row>
-    <row r="310" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="3:5">
       <c r="C310" s="7"/>
       <c r="E310" s="7"/>
     </row>
-    <row r="311" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="3:5">
       <c r="C311" s="7"/>
       <c r="E311" s="7"/>
     </row>
-    <row r="312" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="3:5">
       <c r="C312" s="7"/>
       <c r="E312" s="7"/>
     </row>
-    <row r="313" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="3:5">
       <c r="C313" s="7"/>
       <c r="E313" s="7"/>
     </row>
-    <row r="314" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="3:5">
       <c r="C314" s="7"/>
       <c r="E314" s="7"/>
     </row>
-    <row r="315" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="315" spans="3:5">
       <c r="C315" s="7"/>
       <c r="E315" s="7"/>
     </row>
-    <row r="316" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="3:5">
       <c r="C316" s="7"/>
       <c r="E316" s="7"/>
     </row>
-    <row r="317" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="3:5">
       <c r="C317" s="7"/>
       <c r="E317" s="7"/>
     </row>
-    <row r="318" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="3:5">
       <c r="C318" s="7"/>
       <c r="E318" s="7"/>
     </row>
-    <row r="319" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="3:5">
       <c r="C319" s="7"/>
       <c r="E319" s="7"/>
     </row>
-    <row r="320" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="3:5">
       <c r="C320" s="7"/>
       <c r="E320" s="7"/>
     </row>
-    <row r="321" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="3:5">
       <c r="C321" s="7"/>
       <c r="E321" s="7"/>
     </row>
-    <row r="322" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="3:5">
       <c r="C322" s="7"/>
       <c r="E322" s="7"/>
     </row>
-    <row r="323" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="3:5">
       <c r="C323" s="7"/>
       <c r="E323" s="7"/>
     </row>
-    <row r="324" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="3:5">
       <c r="C324" s="7"/>
       <c r="E324" s="7"/>
     </row>
-    <row r="325" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="3:5">
       <c r="C325" s="7"/>
       <c r="E325" s="7"/>
     </row>
-    <row r="326" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="3:5">
       <c r="C326" s="7"/>
       <c r="E326" s="7"/>
     </row>
-    <row r="327" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="3:5">
       <c r="C327" s="7"/>
       <c r="E327" s="7"/>
     </row>
-    <row r="328" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="3:5">
       <c r="C328" s="7"/>
       <c r="E328" s="7"/>
     </row>
-    <row r="329" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="3:5">
       <c r="C329" s="7"/>
       <c r="E329" s="7"/>
     </row>
-    <row r="330" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="3:5">
       <c r="C330" s="7"/>
       <c r="E330" s="7"/>
     </row>
-    <row r="331" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="3:5">
       <c r="C331" s="7"/>
       <c r="E331" s="7"/>
     </row>
-    <row r="332" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="3:5">
       <c r="C332" s="7"/>
       <c r="E332" s="7"/>
     </row>
-    <row r="333" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="3:5">
       <c r="C333" s="7"/>
       <c r="E333" s="7"/>
     </row>
-    <row r="334" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="3:5">
       <c r="C334" s="7"/>
       <c r="E334" s="7"/>
     </row>
-    <row r="335" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="3:5">
       <c r="C335" s="7"/>
       <c r="E335" s="7"/>
     </row>
-    <row r="336" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="3:5">
       <c r="C336" s="7"/>
       <c r="E336" s="7"/>
     </row>
-    <row r="337" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="3:5">
       <c r="C337" s="7"/>
       <c r="E337" s="7"/>
     </row>
-    <row r="338" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="3:5">
       <c r="C338" s="7"/>
       <c r="E338" s="7"/>
     </row>
-    <row r="339" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="3:5">
       <c r="C339" s="7"/>
       <c r="E339" s="7"/>
     </row>
-    <row r="340" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="3:5">
       <c r="C340" s="7"/>
       <c r="E340" s="7"/>
     </row>
-    <row r="341" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="3:5">
       <c r="C341" s="7"/>
       <c r="E341" s="7"/>
     </row>
-    <row r="342" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="342" spans="3:5">
       <c r="C342" s="7"/>
       <c r="E342" s="7"/>
     </row>
-    <row r="343" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="343" spans="3:5">
       <c r="C343" s="7"/>
       <c r="E343" s="7"/>
     </row>
-    <row r="344" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="344" spans="3:5">
       <c r="C344" s="7"/>
       <c r="E344" s="7"/>
     </row>
-    <row r="345" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="345" spans="3:5">
       <c r="C345" s="7"/>
       <c r="E345" s="7"/>
     </row>
-    <row r="346" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="346" spans="3:5">
       <c r="C346" s="7"/>
       <c r="E346" s="7"/>
     </row>
-    <row r="347" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="347" spans="3:5">
       <c r="C347" s="7"/>
       <c r="E347" s="7"/>
     </row>
-    <row r="348" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="348" spans="3:5">
       <c r="C348" s="7"/>
       <c r="E348" s="7"/>
     </row>
-    <row r="349" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="349" spans="3:5">
       <c r="C349" s="7"/>
       <c r="E349" s="7"/>
     </row>
-    <row r="350" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="350" spans="3:5">
       <c r="C350" s="7"/>
       <c r="E350" s="7"/>
     </row>
-    <row r="351" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="351" spans="3:5">
       <c r="C351" s="7"/>
       <c r="E351" s="7"/>
     </row>
-    <row r="352" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="352" spans="3:5">
       <c r="C352" s="7"/>
       <c r="E352" s="7"/>
     </row>
-    <row r="353" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="353" spans="3:5">
       <c r="C353" s="7"/>
       <c r="E353" s="7"/>
     </row>
-    <row r="354" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="354" spans="3:5">
       <c r="C354" s="7"/>
       <c r="E354" s="7"/>
     </row>
-    <row r="355" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="355" spans="3:5">
       <c r="C355" s="7"/>
       <c r="E355" s="7"/>
     </row>
-    <row r="356" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="356" spans="3:5">
       <c r="C356" s="7"/>
       <c r="E356" s="7"/>
     </row>
-    <row r="357" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="357" spans="3:5">
       <c r="C357" s="7"/>
       <c r="E357" s="7"/>
     </row>
-    <row r="358" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="358" spans="3:5">
       <c r="C358" s="7"/>
       <c r="E358" s="7"/>
     </row>
-    <row r="359" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="359" spans="3:5">
       <c r="C359" s="7"/>
       <c r="E359" s="7"/>
     </row>
-    <row r="360" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="360" spans="3:5">
       <c r="C360" s="7"/>
       <c r="E360" s="7"/>
     </row>
-    <row r="361" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="361" spans="3:5">
       <c r="C361" s="7"/>
       <c r="E361" s="7"/>
     </row>
-    <row r="362" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="362" spans="3:5">
       <c r="C362" s="7"/>
       <c r="E362" s="7"/>
     </row>
-    <row r="363" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="363" spans="3:5">
       <c r="C363" s="7"/>
       <c r="E363" s="7"/>
     </row>
-    <row r="364" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="364" spans="3:5">
       <c r="C364" s="7"/>
       <c r="E364" s="7"/>
     </row>
-    <row r="365" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="365" spans="3:5">
       <c r="C365" s="7"/>
       <c r="E365" s="7"/>
     </row>
-    <row r="366" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="366" spans="3:5">
       <c r="C366" s="7"/>
       <c r="E366" s="7"/>
     </row>
-    <row r="367" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="3:5">
       <c r="C367" s="7"/>
       <c r="E367" s="7"/>
     </row>
-    <row r="368" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="368" spans="3:5">
       <c r="C368" s="7"/>
       <c r="E368" s="7"/>
     </row>
-    <row r="369" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="369" spans="3:5">
       <c r="C369" s="7"/>
       <c r="E369" s="7"/>
     </row>
-    <row r="370" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="3:5">
       <c r="C370" s="7"/>
       <c r="E370" s="7"/>
     </row>
-    <row r="371" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="371" spans="3:5">
       <c r="C371" s="7"/>
       <c r="E371" s="7"/>
     </row>
-    <row r="372" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="372" spans="3:5">
       <c r="C372" s="7"/>
       <c r="E372" s="7"/>
     </row>
-    <row r="373" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="373" spans="3:5">
       <c r="C373" s="7"/>
       <c r="E373" s="7"/>
     </row>
-    <row r="374" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="374" spans="3:5">
       <c r="C374" s="7"/>
       <c r="E374" s="7"/>
     </row>
-    <row r="375" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="375" spans="3:5">
       <c r="C375" s="7"/>
       <c r="E375" s="7"/>
     </row>
-    <row r="376" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="376" spans="3:5">
       <c r="C376" s="7"/>
       <c r="E376" s="7"/>
     </row>
-    <row r="377" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="377" spans="3:5">
       <c r="C377" s="7"/>
       <c r="E377" s="7"/>
     </row>
-    <row r="378" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="378" spans="3:5">
       <c r="C378" s="7"/>
       <c r="E378" s="7"/>
     </row>
-    <row r="379" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="379" spans="3:5">
       <c r="C379" s="7"/>
       <c r="E379" s="7"/>
     </row>
-    <row r="380" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="380" spans="3:5">
       <c r="C380" s="7"/>
       <c r="E380" s="7"/>
     </row>
-    <row r="381" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="381" spans="3:5">
       <c r="C381" s="7"/>
       <c r="E381" s="7"/>
     </row>
-    <row r="382" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="382" spans="3:5">
       <c r="C382" s="7"/>
       <c r="E382" s="7"/>
     </row>
-    <row r="383" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="383" spans="3:5">
       <c r="C383" s="7"/>
       <c r="E383" s="7"/>
     </row>
-    <row r="384" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="384" spans="3:5">
       <c r="C384" s="7"/>
       <c r="E384" s="7"/>
     </row>
-    <row r="385" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="385" spans="3:5">
       <c r="C385" s="7"/>
       <c r="E385" s="7"/>
     </row>
-    <row r="386" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="386" spans="3:5">
       <c r="C386" s="7"/>
       <c r="E386" s="7"/>
     </row>
-    <row r="387" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="387" spans="3:5">
       <c r="C387" s="7"/>
       <c r="E387" s="7"/>
     </row>
-    <row r="388" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="388" spans="3:5">
       <c r="C388" s="7"/>
       <c r="E388" s="7"/>
     </row>
-    <row r="389" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="389" spans="3:5">
       <c r="C389" s="7"/>
       <c r="E389" s="7"/>
     </row>
-    <row r="390" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="390" spans="3:5">
       <c r="C390" s="7"/>
       <c r="E390" s="7"/>
     </row>
-    <row r="391" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="391" spans="3:5">
       <c r="C391" s="7"/>
       <c r="E391" s="7"/>
     </row>
-    <row r="392" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="392" spans="3:5">
       <c r="C392" s="7"/>
       <c r="E392" s="7"/>
     </row>
-    <row r="393" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="393" spans="3:5">
       <c r="C393" s="7"/>
       <c r="E393" s="7"/>
     </row>
-    <row r="394" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="394" spans="3:5">
       <c r="C394" s="7"/>
       <c r="E394" s="7"/>
     </row>
-    <row r="395" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="395" spans="3:5">
       <c r="C395" s="7"/>
       <c r="E395" s="7"/>
     </row>
-    <row r="396" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="396" spans="3:5">
       <c r="C396" s="7"/>
       <c r="E396" s="7"/>
     </row>
-    <row r="397" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="397" spans="3:5">
       <c r="C397" s="7"/>
       <c r="E397" s="7"/>
     </row>
-    <row r="398" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="398" spans="3:5">
       <c r="C398" s="7"/>
       <c r="E398" s="7"/>
     </row>
-    <row r="399" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="399" spans="3:5">
       <c r="C399" s="7"/>
       <c r="E399" s="7"/>
     </row>
-    <row r="400" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="400" spans="3:5">
       <c r="C400" s="7"/>
       <c r="E400" s="7"/>
     </row>
-    <row r="401" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="401" spans="3:5">
       <c r="C401" s="7"/>
       <c r="E401" s="7"/>
     </row>
-    <row r="402" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="402" spans="3:5">
       <c r="C402" s="7"/>
       <c r="E402" s="7"/>
     </row>
-    <row r="403" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="403" spans="3:5">
       <c r="C403" s="7"/>
       <c r="E403" s="7"/>
     </row>
-    <row r="404" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="404" spans="3:5">
       <c r="C404" s="7"/>
       <c r="E404" s="7"/>
     </row>
-    <row r="405" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="405" spans="3:5">
       <c r="C405" s="7"/>
       <c r="E405" s="7"/>
     </row>
-    <row r="406" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="406" spans="3:5">
       <c r="C406" s="7"/>
       <c r="E406" s="7"/>
     </row>
-    <row r="407" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="407" spans="3:5">
       <c r="C407" s="7"/>
       <c r="E407" s="7"/>
     </row>
-    <row r="408" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="408" spans="3:5">
       <c r="C408" s="7"/>
       <c r="E408" s="7"/>
     </row>
-    <row r="409" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="409" spans="3:5">
       <c r="C409" s="7"/>
       <c r="E409" s="7"/>
     </row>
-    <row r="410" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="410" spans="3:5">
       <c r="C410" s="7"/>
       <c r="E410" s="7"/>
     </row>
-    <row r="411" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="411" spans="3:5">
       <c r="C411" s="7"/>
       <c r="E411" s="7"/>
     </row>
-    <row r="412" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="412" spans="3:5">
       <c r="C412" s="7"/>
       <c r="E412" s="7"/>
     </row>
-    <row r="413" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="413" spans="3:5">
       <c r="C413" s="7"/>
       <c r="E413" s="7"/>
     </row>
-    <row r="414" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="414" spans="3:5">
       <c r="C414" s="7"/>
       <c r="E414" s="7"/>
     </row>
-    <row r="415" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="415" spans="3:5">
       <c r="C415" s="7"/>
       <c r="E415" s="7"/>
     </row>
-    <row r="416" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="416" spans="3:5">
       <c r="C416" s="7"/>
       <c r="E416" s="7"/>
     </row>
-    <row r="417" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="417" spans="3:5">
       <c r="C417" s="7"/>
       <c r="E417" s="7"/>
     </row>
-    <row r="418" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="418" spans="3:5">
       <c r="C418" s="7"/>
       <c r="E418" s="7"/>
     </row>
-    <row r="419" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="419" spans="3:5">
       <c r="C419" s="7"/>
       <c r="E419" s="7"/>
     </row>
-    <row r="420" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="420" spans="3:5">
       <c r="C420" s="7"/>
       <c r="E420" s="7"/>
     </row>
-    <row r="421" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="421" spans="3:5">
       <c r="C421" s="7"/>
       <c r="E421" s="7"/>
     </row>
-    <row r="422" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="422" spans="3:5">
       <c r="C422" s="7"/>
       <c r="E422" s="7"/>
     </row>
-    <row r="423" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="423" spans="3:5">
       <c r="C423" s="7"/>
       <c r="E423" s="7"/>
     </row>
-    <row r="424" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="424" spans="3:5">
       <c r="C424" s="7"/>
       <c r="E424" s="7"/>
     </row>
-    <row r="425" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="425" spans="3:5">
       <c r="C425" s="7"/>
       <c r="E425" s="7"/>
     </row>
-    <row r="426" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="426" spans="3:5">
       <c r="C426" s="7"/>
       <c r="E426" s="7"/>
     </row>
-    <row r="427" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="427" spans="3:5">
       <c r="C427" s="7"/>
       <c r="E427" s="7"/>
     </row>
-    <row r="428" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="428" spans="3:5">
       <c r="C428" s="7"/>
       <c r="E428" s="7"/>
     </row>
-    <row r="429" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="429" spans="3:5">
       <c r="C429" s="7"/>
       <c r="E429" s="7"/>
     </row>
-    <row r="430" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="430" spans="3:5">
       <c r="C430" s="7"/>
       <c r="E430" s="7"/>
     </row>
-    <row r="431" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="431" spans="3:5">
       <c r="C431" s="7"/>
       <c r="E431" s="7"/>
     </row>
-    <row r="432" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="432" spans="3:5">
       <c r="C432" s="7"/>
       <c r="E432" s="7"/>
     </row>
-    <row r="433" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="433" spans="3:5">
       <c r="C433" s="7"/>
       <c r="E433" s="7"/>
     </row>
-    <row r="434" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="434" spans="3:5">
       <c r="C434" s="7"/>
       <c r="E434" s="7"/>
     </row>
-    <row r="435" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="435" spans="3:5">
       <c r="C435" s="7"/>
       <c r="E435" s="7"/>
     </row>
-    <row r="436" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="436" spans="3:5">
       <c r="C436" s="7"/>
       <c r="E436" s="7"/>
     </row>
-    <row r="437" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="437" spans="3:5">
       <c r="C437" s="7"/>
       <c r="E437" s="7"/>
     </row>
-    <row r="438" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="438" spans="3:5">
       <c r="C438" s="7"/>
       <c r="E438" s="7"/>
     </row>
-    <row r="439" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="439" spans="3:5">
       <c r="C439" s="7"/>
       <c r="E439" s="7"/>
     </row>
-    <row r="440" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="440" spans="3:5">
       <c r="C440" s="7"/>
       <c r="E440" s="7"/>
     </row>
-    <row r="441" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="441" spans="3:5">
       <c r="C441" s="7"/>
       <c r="E441" s="7"/>
     </row>
-    <row r="442" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="442" spans="3:5">
       <c r="C442" s="7"/>
       <c r="E442" s="7"/>
     </row>
-    <row r="443" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="443" spans="3:5">
       <c r="C443" s="7"/>
       <c r="E443" s="7"/>
     </row>
-    <row r="444" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="444" spans="3:5">
       <c r="C444" s="7"/>
       <c r="E444" s="7"/>
     </row>
-    <row r="445" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="445" spans="3:5">
       <c r="C445" s="7"/>
       <c r="E445" s="7"/>
     </row>
-    <row r="446" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="446" spans="3:5">
       <c r="C446" s="7"/>
       <c r="E446" s="7"/>
     </row>
-    <row r="447" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="447" spans="3:5">
       <c r="C447" s="7"/>
       <c r="E447" s="7"/>
     </row>
-    <row r="448" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="448" spans="3:5">
       <c r="C448" s="7"/>
       <c r="E448" s="7"/>
     </row>
-    <row r="449" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="449" spans="3:5">
       <c r="C449" s="7"/>
       <c r="E449" s="7"/>
     </row>
-    <row r="450" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="450" spans="3:5">
       <c r="C450" s="7"/>
       <c r="E450" s="7"/>
     </row>
-    <row r="451" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="451" spans="3:5">
       <c r="C451" s="7"/>
       <c r="E451" s="7"/>
     </row>
-    <row r="452" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="452" spans="3:5">
       <c r="C452" s="7"/>
       <c r="E452" s="7"/>
     </row>
-    <row r="453" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="453" spans="3:5">
       <c r="C453" s="7"/>
       <c r="E453" s="7"/>
     </row>
-    <row r="454" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="454" spans="3:5">
       <c r="C454" s="7"/>
       <c r="E454" s="7"/>
     </row>
-    <row r="455" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="455" spans="3:5">
       <c r="C455" s="7"/>
       <c r="E455" s="7"/>
     </row>
-    <row r="456" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="456" spans="3:5">
       <c r="C456" s="7"/>
       <c r="E456" s="7"/>
     </row>
-    <row r="457" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="457" spans="3:5">
       <c r="C457" s="7"/>
       <c r="E457" s="7"/>
     </row>
-    <row r="458" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="458" spans="3:5">
       <c r="C458" s="7"/>
       <c r="E458" s="7"/>
     </row>
-    <row r="459" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="459" spans="3:5">
       <c r="C459" s="7"/>
       <c r="E459" s="7"/>
     </row>
-    <row r="460" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="460" spans="3:5">
       <c r="C460" s="7"/>
       <c r="E460" s="7"/>
     </row>
-    <row r="461" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="461" spans="3:5">
       <c r="C461" s="7"/>
       <c r="E461" s="7"/>
     </row>
-    <row r="462" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="462" spans="3:5">
       <c r="C462" s="7"/>
       <c r="E462" s="7"/>
     </row>
-    <row r="463" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="463" spans="3:5">
       <c r="C463" s="7"/>
       <c r="E463" s="7"/>
     </row>
-    <row r="464" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="464" spans="3:5">
       <c r="C464" s="7"/>
       <c r="E464" s="7"/>
     </row>
-    <row r="465" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="465" spans="3:5">
       <c r="C465" s="7"/>
       <c r="E465" s="7"/>
     </row>
-    <row r="466" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="466" spans="3:5">
       <c r="C466" s="7"/>
       <c r="E466" s="7"/>
     </row>
-    <row r="467" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="467" spans="3:5">
       <c r="C467" s="7"/>
       <c r="E467" s="7"/>
     </row>
-    <row r="468" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="468" spans="3:5">
       <c r="C468" s="7"/>
       <c r="E468" s="7"/>
     </row>
-    <row r="469" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="469" spans="3:5">
       <c r="C469" s="7"/>
       <c r="E469" s="7"/>
     </row>
-    <row r="470" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="470" spans="3:5">
       <c r="C470" s="7"/>
       <c r="E470" s="7"/>
     </row>
-    <row r="471" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="471" spans="3:5">
       <c r="C471" s="7"/>
       <c r="E471" s="7"/>
     </row>
-    <row r="472" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="472" spans="3:5">
       <c r="C472" s="7"/>
       <c r="E472" s="7"/>
     </row>
-    <row r="473" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="473" spans="3:5">
       <c r="C473" s="7"/>
       <c r="E473" s="7"/>
     </row>
-    <row r="474" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="474" spans="3:5">
       <c r="C474" s="7"/>
       <c r="E474" s="7"/>
     </row>
-    <row r="475" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="475" spans="3:5">
       <c r="C475" s="7"/>
       <c r="E475" s="7"/>
     </row>
-    <row r="476" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="476" spans="3:5">
       <c r="C476" s="7"/>
       <c r="E476" s="7"/>
     </row>
-    <row r="477" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="477" spans="3:5">
       <c r="C477" s="7"/>
       <c r="E477" s="7"/>
     </row>
-    <row r="478" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="478" spans="3:5">
       <c r="C478" s="7"/>
       <c r="E478" s="7"/>
     </row>
-    <row r="479" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="479" spans="3:5">
       <c r="C479" s="7"/>
       <c r="E479" s="7"/>
     </row>
-    <row r="480" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="480" spans="3:5">
       <c r="C480" s="7"/>
       <c r="E480" s="7"/>
     </row>
-    <row r="481" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="481" spans="3:5">
       <c r="C481" s="7"/>
       <c r="E481" s="7"/>
     </row>
-    <row r="482" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="482" spans="3:5">
       <c r="C482" s="7"/>
       <c r="E482" s="7"/>
     </row>
-    <row r="483" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="483" spans="3:5">
       <c r="C483" s="7"/>
       <c r="E483" s="7"/>
     </row>
-    <row r="484" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="484" spans="3:5">
       <c r="C484" s="7"/>
       <c r="E484" s="7"/>
     </row>
-    <row r="485" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="485" spans="3:5">
       <c r="C485" s="7"/>
       <c r="E485" s="7"/>
     </row>
-    <row r="486" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="486" spans="3:5">
       <c r="C486" s="7"/>
       <c r="E486" s="7"/>
     </row>
-    <row r="487" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="487" spans="3:5">
       <c r="C487" s="7"/>
       <c r="E487" s="7"/>
     </row>
-    <row r="488" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="488" spans="3:5">
       <c r="C488" s="7"/>
       <c r="E488" s="7"/>
     </row>
-    <row r="489" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="489" spans="3:5">
       <c r="C489" s="7"/>
       <c r="E489" s="7"/>
     </row>
-    <row r="490" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="490" spans="3:5">
       <c r="C490" s="7"/>
       <c r="E490" s="7"/>
     </row>
-    <row r="491" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="491" spans="3:5">
       <c r="C491" s="7"/>
       <c r="E491" s="7"/>
     </row>
-    <row r="492" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="492" spans="3:5">
       <c r="C492" s="7"/>
       <c r="E492" s="7"/>
     </row>
-    <row r="493" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="493" spans="3:5">
       <c r="C493" s="7"/>
       <c r="E493" s="7"/>
     </row>
-    <row r="494" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="494" spans="3:5">
       <c r="C494" s="7"/>
       <c r="E494" s="7"/>
     </row>
-    <row r="495" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="495" spans="3:5">
       <c r="C495" s="7"/>
       <c r="E495" s="7"/>
     </row>
-    <row r="496" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="496" spans="3:5">
       <c r="C496" s="7"/>
       <c r="E496" s="7"/>
     </row>
-    <row r="497" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="497" spans="3:5">
       <c r="C497" s="7"/>
       <c r="E497" s="7"/>
     </row>
-    <row r="498" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="498" spans="3:5">
       <c r="C498" s="7"/>
       <c r="E498" s="7"/>
     </row>
-    <row r="499" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="499" spans="3:5">
       <c r="C499" s="7"/>
       <c r="E499" s="7"/>
     </row>
-    <row r="500" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="500" spans="3:5">
       <c r="C500" s="7"/>
       <c r="E500" s="7"/>
     </row>
-    <row r="501" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="501" spans="3:5">
       <c r="C501" s="7"/>
       <c r="E501" s="7"/>
     </row>
-    <row r="502" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="502" spans="3:5">
       <c r="C502" s="7"/>
       <c r="E502" s="7"/>
     </row>
-    <row r="503" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="503" spans="3:5">
       <c r="C503" s="7"/>
       <c r="E503" s="7"/>
     </row>
-    <row r="504" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="504" spans="3:5">
       <c r="C504" s="7"/>
       <c r="E504" s="7"/>
     </row>
-    <row r="505" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="505" spans="3:5">
       <c r="C505" s="7"/>
       <c r="E505" s="7"/>
     </row>
-    <row r="506" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="506" spans="3:5">
       <c r="C506" s="7"/>
       <c r="E506" s="7"/>
     </row>
-    <row r="507" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="507" spans="3:5">
       <c r="C507" s="7"/>
       <c r="E507" s="7"/>
     </row>
-    <row r="508" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="508" spans="3:5">
       <c r="C508" s="7"/>
       <c r="E508" s="7"/>
     </row>
-    <row r="509" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="509" spans="3:5">
       <c r="C509" s="7"/>
       <c r="E509" s="7"/>
     </row>
-    <row r="510" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="510" spans="3:5">
       <c r="C510" s="7"/>
       <c r="E510" s="7"/>
     </row>
-    <row r="511" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="511" spans="3:5">
       <c r="C511" s="7"/>
       <c r="E511" s="7"/>
     </row>
-    <row r="512" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="512" spans="3:5">
       <c r="C512" s="7"/>
       <c r="E512" s="7"/>
     </row>
-    <row r="513" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="513" spans="3:5">
       <c r="C513" s="7"/>
       <c r="E513" s="7"/>
     </row>
-    <row r="514" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="514" spans="3:5">
       <c r="C514" s="7"/>
       <c r="E514" s="7"/>
     </row>
-    <row r="515" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="515" spans="3:5">
       <c r="C515" s="7"/>
       <c r="E515" s="7"/>
     </row>
-    <row r="516" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="516" spans="3:5">
       <c r="C516" s="7"/>
       <c r="E516" s="7"/>
     </row>
-    <row r="517" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="517" spans="3:5">
       <c r="C517" s="7"/>
       <c r="E517" s="7"/>
     </row>
-    <row r="518" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="518" spans="3:5">
       <c r="C518" s="7"/>
       <c r="E518" s="7"/>
     </row>
-    <row r="519" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="519" spans="3:5">
       <c r="C519" s="7"/>
       <c r="E519" s="7"/>
     </row>
-    <row r="520" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="520" spans="3:5">
       <c r="C520" s="7"/>
       <c r="E520" s="7"/>
     </row>
-    <row r="521" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="521" spans="3:5">
       <c r="C521" s="7"/>
       <c r="E521" s="7"/>
     </row>
-    <row r="522" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="522" spans="3:5">
       <c r="C522" s="7"/>
       <c r="E522" s="7"/>
     </row>
-    <row r="523" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="523" spans="3:5">
       <c r="C523" s="7"/>
       <c r="E523" s="7"/>
     </row>
-    <row r="524" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="524" spans="3:5">
       <c r="C524" s="7"/>
       <c r="E524" s="7"/>
     </row>
-    <row r="525" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="525" spans="3:5">
       <c r="C525" s="7"/>
       <c r="E525" s="7"/>
     </row>
-    <row r="526" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="526" spans="3:5">
       <c r="C526" s="7"/>
       <c r="E526" s="7"/>
     </row>
-    <row r="527" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="527" spans="3:5">
       <c r="C527" s="7"/>
       <c r="E527" s="7"/>
     </row>
-    <row r="528" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="528" spans="3:5">
       <c r="C528" s="7"/>
       <c r="E528" s="7"/>
     </row>
-    <row r="529" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="529" spans="3:5">
       <c r="C529" s="7"/>
       <c r="E529" s="7"/>
     </row>
-    <row r="530" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="530" spans="3:5">
       <c r="C530" s="7"/>
       <c r="E530" s="7"/>
     </row>
-    <row r="531" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="531" spans="3:5">
       <c r="C531" s="7"/>
       <c r="E531" s="7"/>
     </row>
-    <row r="532" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="532" spans="3:5">
       <c r="C532" s="7"/>
       <c r="E532" s="7"/>
     </row>
-    <row r="533" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="533" spans="3:5">
       <c r="C533" s="7"/>
       <c r="E533" s="7"/>
     </row>
-    <row r="534" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="534" spans="3:5">
       <c r="C534" s="7"/>
       <c r="E534" s="7"/>
     </row>
-    <row r="535" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="535" spans="3:5">
       <c r="C535" s="7"/>
       <c r="E535" s="7"/>
     </row>
-    <row r="536" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="536" spans="3:5">
       <c r="C536" s="7"/>
       <c r="E536" s="7"/>
     </row>
-    <row r="537" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="537" spans="3:5">
       <c r="C537" s="7"/>
       <c r="E537" s="7"/>
     </row>
-    <row r="538" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="538" spans="3:5">
       <c r="C538" s="7"/>
       <c r="E538" s="7"/>
     </row>
-    <row r="539" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="539" spans="3:5">
       <c r="C539" s="7"/>
       <c r="E539" s="7"/>
     </row>
-    <row r="540" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="540" spans="3:5">
       <c r="C540" s="7"/>
       <c r="E540" s="7"/>
     </row>
-    <row r="541" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="541" spans="3:5">
       <c r="C541" s="7"/>
       <c r="E541" s="7"/>
     </row>
-    <row r="542" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="542" spans="3:5">
       <c r="C542" s="7"/>
       <c r="E542" s="7"/>
     </row>
-    <row r="543" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="543" spans="3:5">
       <c r="C543" s="7"/>
       <c r="E543" s="7"/>
     </row>
-    <row r="544" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="544" spans="3:5">
       <c r="C544" s="7"/>
       <c r="E544" s="7"/>
     </row>
-    <row r="545" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="545" spans="3:5">
       <c r="C545" s="7"/>
       <c r="E545" s="7"/>
     </row>
-    <row r="546" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="546" spans="3:5">
       <c r="C546" s="7"/>
       <c r="E546" s="7"/>
     </row>
-    <row r="547" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="547" spans="3:5">
       <c r="C547" s="7"/>
       <c r="E547" s="7"/>
     </row>
-    <row r="548" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="548" spans="3:5">
       <c r="C548" s="7"/>
       <c r="E548" s="7"/>
     </row>
-    <row r="549" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="549" spans="3:5">
       <c r="C549" s="7"/>
       <c r="E549" s="7"/>
     </row>
-    <row r="550" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="550" spans="3:5">
       <c r="C550" s="7"/>
       <c r="E550" s="7"/>
     </row>
-    <row r="551" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="551" spans="3:5">
       <c r="C551" s="7"/>
       <c r="E551" s="7"/>
     </row>
-    <row r="552" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="552" spans="3:5">
       <c r="C552" s="7"/>
       <c r="E552" s="7"/>
     </row>
-    <row r="553" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="553" spans="3:5">
       <c r="C553" s="7"/>
       <c r="E553" s="7"/>
     </row>
-    <row r="554" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="554" spans="3:5">
       <c r="C554" s="7"/>
       <c r="E554" s="7"/>
     </row>
-    <row r="555" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="555" spans="3:5">
       <c r="C555" s="7"/>
       <c r="E555" s="7"/>
     </row>
-    <row r="556" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="556" spans="3:5">
       <c r="C556" s="7"/>
       <c r="E556" s="7"/>
     </row>
-    <row r="557" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="557" spans="3:5">
       <c r="C557" s="7"/>
       <c r="E557" s="7"/>
     </row>
-    <row r="558" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="558" spans="3:5">
       <c r="C558" s="7"/>
       <c r="E558" s="7"/>
     </row>
-    <row r="559" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="559" spans="3:5">
       <c r="C559" s="7"/>
       <c r="E559" s="7"/>
     </row>
-    <row r="560" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="560" spans="3:5">
       <c r="C560" s="7"/>
       <c r="E560" s="7"/>
     </row>
-    <row r="561" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="561" spans="3:5">
       <c r="C561" s="7"/>
       <c r="E561" s="7"/>
     </row>
-    <row r="562" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="562" spans="3:5">
       <c r="C562" s="7"/>
       <c r="E562" s="7"/>
     </row>
-    <row r="563" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="563" spans="3:5">
       <c r="C563" s="7"/>
       <c r="E563" s="7"/>
     </row>
-    <row r="564" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="564" spans="3:5">
       <c r="C564" s="7"/>
       <c r="E564" s="7"/>
     </row>
-    <row r="565" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="565" spans="3:5">
       <c r="C565" s="7"/>
       <c r="E565" s="7"/>
     </row>
-    <row r="566" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="566" spans="3:5">
       <c r="C566" s="7"/>
       <c r="E566" s="7"/>
     </row>
-    <row r="567" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="567" spans="3:5">
       <c r="C567" s="7"/>
       <c r="E567" s="7"/>
     </row>
-    <row r="568" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="568" spans="3:5">
       <c r="C568" s="7"/>
       <c r="E568" s="7"/>
     </row>
-    <row r="569" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="569" spans="3:5">
       <c r="C569" s="7"/>
       <c r="E569" s="7"/>
     </row>
-    <row r="570" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="570" spans="3:5">
       <c r="C570" s="7"/>
       <c r="E570" s="7"/>
     </row>
-    <row r="571" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="571" spans="3:5">
       <c r="C571" s="7"/>
       <c r="E571" s="7"/>
     </row>
-    <row r="572" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="572" spans="3:5">
       <c r="C572" s="7"/>
       <c r="E572" s="7"/>
     </row>
-    <row r="573" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="573" spans="3:5">
       <c r="C573" s="7"/>
       <c r="E573" s="7"/>
     </row>
-    <row r="574" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="574" spans="3:5">
       <c r="C574" s="7"/>
       <c r="E574" s="7"/>
     </row>
-    <row r="575" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="575" spans="3:5">
       <c r="C575" s="7"/>
       <c r="E575" s="7"/>
     </row>
-    <row r="576" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="576" spans="3:5">
       <c r="C576" s="7"/>
       <c r="E576" s="7"/>
     </row>
-    <row r="577" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="577" spans="3:5">
       <c r="C577" s="7"/>
       <c r="E577" s="7"/>
     </row>
-    <row r="578" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="578" spans="3:5">
       <c r="C578" s="7"/>
       <c r="E578" s="7"/>
     </row>
-    <row r="579" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="579" spans="3:5">
       <c r="C579" s="7"/>
       <c r="E579" s="7"/>
     </row>
-    <row r="580" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="580" spans="3:5">
       <c r="C580" s="7"/>
       <c r="E580" s="7"/>
     </row>
-    <row r="581" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="581" spans="3:5">
       <c r="C581" s="7"/>
       <c r="E581" s="7"/>
     </row>
-    <row r="582" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="582" spans="3:5">
       <c r="C582" s="7"/>
       <c r="E582" s="7"/>
     </row>

</xml_diff>

<commit_message>
Update ATP with updated criterion
</commit_message>
<xml_diff>
--- a/etc/Acceptance Test Plan.xlsx
+++ b/etc/Acceptance Test Plan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phine\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phine\OneDrive\code2\swen\project\team-project-2251-swen-261-05-2-goated\etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F63D7C-8B03-43E3-9781-0E14869E3D3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD2EE67F-08D5-4A77-A06D-A8B6F5374D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Test Plan" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Plan'!$G$1:$G$1000</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Plan'!$G$1:$G$1002</definedName>
   </definedNames>
   <calcPr calcId="0" concurrentCalc="0"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="124">
   <si>
     <t>Instructions</t>
   </si>
@@ -300,9 +300,6 @@
     <t>**Given** I am logged out **when** I try to view any pages requiring an account (any page but Login and Homepage) **then** I am redirected to the login.</t>
   </si>
   <si>
-    <t>As a owner I want to have all tabs located in a dropdown menu so that the website looks better.</t>
-  </si>
-  <si>
     <t>**Given** I am logged in **when** I click on the dropdown menu**then** I see the tab buttons.</t>
   </si>
   <si>
@@ -386,6 +383,30 @@
   <si>
     <t>MM, CM 11/6/2025 Can't go to homepage as a logged in user. Loggin page has login button, not needs</t>
   </si>
+  <si>
+    <t>**Given** I am logged in **when** I go to the thanks tab **then** I should see the number of needs fulfilled in the listed timeframes</t>
+  </si>
+  <si>
+    <t>As a User I want to see how many needs have been checked out in the past day, week, month, etc so that I can get interesting statistics.</t>
+  </si>
+  <si>
+    <t>As a User I want to see the ratio of fulfilled vs unfulfilled needs so that I can get statistics.</t>
+  </si>
+  <si>
+    <t>**Given** I am logged in **when** I go to the thanks tab **then** I should see a pie chart showing the ratio of fulfilled and unfulfilled needs</t>
+  </si>
+  <si>
+    <t>Given I am logged in, when I go to the home page then I should be redirected to the needs page with my current saved login.</t>
+  </si>
+  <si>
+    <t>AC has been changed.</t>
+  </si>
+  <si>
+    <t>**Given** I am logged in **when** I view any page **then** I see the tab buttons.</t>
+  </si>
+  <si>
+    <t>As a user I want to have all tabs located in a navigation menu so that the website looks better.</t>
+  </si>
 </sst>
 </file>
 
@@ -440,7 +461,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -457,11 +478,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -498,6 +539,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3784,7 +3834,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z1000"/>
+  <dimension ref="A1:Z1002"/>
   <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -3798,7 +3848,7 @@
     <col min="9" max="26" width="10.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>6</v>
       </c>
@@ -3861,7 +3911,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I2" s="10"/>
       <c r="J2" s="10"/>
@@ -3899,7 +3949,7 @@
         <v>14</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I3" s="10"/>
       <c r="J3" s="10"/>
@@ -3939,7 +3989,7 @@
         <v>14</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I4" s="10"/>
       <c r="J4" s="10"/>
@@ -3979,7 +4029,7 @@
         <v>14</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
@@ -4017,7 +4067,7 @@
         <v>14</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
@@ -4057,7 +4107,7 @@
         <v>14</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
@@ -4097,7 +4147,7 @@
         <v>14</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
@@ -4135,7 +4185,7 @@
         <v>14</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
@@ -4175,7 +4225,7 @@
         <v>14</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
@@ -4213,7 +4263,7 @@
         <v>14</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
@@ -4251,7 +4301,7 @@
         <v>14</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
@@ -4291,7 +4341,7 @@
         <v>14</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
@@ -4331,7 +4381,7 @@
         <v>14</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
@@ -4369,7 +4419,7 @@
         <v>14</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I15" s="10"/>
       <c r="J15" s="10"/>
@@ -4409,7 +4459,7 @@
         <v>14</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
@@ -4447,7 +4497,7 @@
         <v>14</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
@@ -4487,7 +4537,7 @@
         <v>14</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I18" s="10"/>
       <c r="J18" s="10"/>
@@ -4525,7 +4575,7 @@
         <v>14</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I19" s="10"/>
       <c r="J19" s="10"/>
@@ -4563,7 +4613,7 @@
         <v>14</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I20" s="10"/>
       <c r="J20" s="10"/>
@@ -4603,7 +4653,7 @@
         <v>14</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I21" s="10"/>
       <c r="J21" s="10"/>
@@ -4641,7 +4691,7 @@
         <v>14</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I22" s="10"/>
       <c r="J22" s="10"/>
@@ -4679,7 +4729,7 @@
         <v>14</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I23" s="10"/>
       <c r="J23" s="10"/>
@@ -4719,7 +4769,7 @@
         <v>14</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I24" s="10"/>
       <c r="J24" s="10"/>
@@ -4757,7 +4807,7 @@
         <v>14</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I25" s="10"/>
       <c r="J25" s="10"/>
@@ -4797,7 +4847,7 @@
         <v>14</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I26" s="10"/>
       <c r="J26" s="10"/>
@@ -4835,7 +4885,7 @@
         <v>14</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I27" s="10"/>
       <c r="J27" s="10"/>
@@ -4875,7 +4925,7 @@
         <v>14</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I28" s="10"/>
       <c r="J28" s="10"/>
@@ -4897,8 +4947,8 @@
       <c r="Z28" s="10"/>
     </row>
     <row r="29" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11" t="s">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15" t="s">
         <v>61</v>
       </c>
       <c r="C29" s="9" t="s">
@@ -4908,12 +4958,14 @@
         <v>62</v>
       </c>
       <c r="E29" s="9"/>
-      <c r="F29" s="2"/>
+      <c r="F29" s="2" t="s">
+        <v>121</v>
+      </c>
       <c r="G29" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I29" s="10"/>
       <c r="J29" s="10"/>
@@ -4934,27 +4986,17 @@
       <c r="Y29" s="10"/>
       <c r="Z29" s="10"/>
     </row>
-    <row r="30" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A30" s="12" t="s">
-        <v>63</v>
+    <row r="30" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="11"/>
+      <c r="B30" s="11" t="s">
+        <v>120</v>
       </c>
-      <c r="B30" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="C30" s="9"/>
+      <c r="D30" s="2"/>
       <c r="E30" s="9"/>
       <c r="F30" s="2"/>
-      <c r="G30" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>111</v>
-      </c>
+      <c r="G30" s="9"/>
+      <c r="H30" s="2"/>
       <c r="I30" s="10"/>
       <c r="J30" s="10"/>
       <c r="K30" s="10"/>
@@ -4974,22 +5016,26 @@
       <c r="Y30" s="10"/>
       <c r="Z30" s="10"/>
     </row>
-    <row r="31" spans="1:26" ht="93" x14ac:dyDescent="0.35">
-      <c r="A31" s="13" t="s">
-        <v>65</v>
+    <row r="31" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="12" t="s">
+        <v>63</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>66</v>
+      <c r="B31" s="11" t="s">
+        <v>64</v>
       </c>
-      <c r="C31" s="9"/>
-      <c r="D31" s="2"/>
+      <c r="C31" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="E31" s="9"/>
       <c r="F31" s="2"/>
       <c r="G31" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I31" s="10"/>
       <c r="J31" s="10"/>
@@ -5011,9 +5057,11 @@
       <c r="Z31" s="10"/>
     </row>
     <row r="32" spans="1:26" ht="93" x14ac:dyDescent="0.35">
-      <c r="A32" s="12"/>
-      <c r="B32" s="11" t="s">
-        <v>67</v>
+      <c r="A32" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>66</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="2"/>
@@ -5023,7 +5071,7 @@
         <v>14</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I32" s="10"/>
       <c r="J32" s="10"/>
@@ -5044,12 +5092,10 @@
       <c r="Y32" s="10"/>
       <c r="Z32" s="10"/>
     </row>
-    <row r="33" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>69</v>
+    <row r="33" spans="1:26" ht="93.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="12"/>
+      <c r="B33" s="11" t="s">
+        <v>67</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="2"/>
@@ -5059,7 +5105,7 @@
         <v>14</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I33" s="10"/>
       <c r="J33" s="10"/>
@@ -5080,10 +5126,12 @@
       <c r="Y33" s="10"/>
       <c r="Z33" s="10"/>
     </row>
-    <row r="34" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A34" s="11"/>
-      <c r="B34" s="11" t="s">
-        <v>70</v>
+    <row r="34" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>69</v>
       </c>
       <c r="C34" s="9"/>
       <c r="D34" s="2"/>
@@ -5093,7 +5141,7 @@
         <v>14</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I34" s="10"/>
       <c r="J34" s="10"/>
@@ -5114,12 +5162,10 @@
       <c r="Y34" s="10"/>
       <c r="Z34" s="10"/>
     </row>
-    <row r="35" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A35" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>72</v>
+    <row r="35" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="11"/>
+      <c r="B35" s="11" t="s">
+        <v>70</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="2"/>
@@ -5129,7 +5175,7 @@
         <v>14</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I35" s="10"/>
       <c r="J35" s="10"/>
@@ -5150,10 +5196,12 @@
       <c r="Y35" s="10"/>
       <c r="Z35" s="10"/>
     </row>
-    <row r="36" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11" t="s">
-        <v>73</v>
+    <row r="36" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>72</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="2"/>
@@ -5163,7 +5211,7 @@
         <v>14</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I36" s="10"/>
       <c r="J36" s="10"/>
@@ -5184,12 +5232,10 @@
       <c r="Y36" s="10"/>
       <c r="Z36" s="10"/>
     </row>
-    <row r="37" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A37" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>75</v>
+    <row r="37" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="11"/>
+      <c r="B37" s="11" t="s">
+        <v>73</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="2"/>
@@ -5199,7 +5245,7 @@
         <v>14</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I37" s="10"/>
       <c r="J37" s="10"/>
@@ -5221,17 +5267,21 @@
       <c r="Z37" s="10"/>
     </row>
     <row r="38" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11" t="s">
-        <v>76</v>
+      <c r="A38" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>75</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="2"/>
       <c r="E38" s="9"/>
       <c r="F38" s="2"/>
-      <c r="G38" s="9"/>
+      <c r="G38" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="H38" s="2" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="I38" s="10"/>
       <c r="J38" s="10"/>
@@ -5252,22 +5302,18 @@
       <c r="Y38" s="10"/>
       <c r="Z38" s="10"/>
     </row>
-    <row r="39" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A39" s="11" t="s">
-        <v>78</v>
-      </c>
+    <row r="39" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="11"/>
       <c r="B39" s="11" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C39" s="9"/>
       <c r="D39" s="2"/>
       <c r="E39" s="9"/>
       <c r="F39" s="2"/>
-      <c r="G39" s="9" t="s">
-        <v>14</v>
-      </c>
+      <c r="G39" s="9"/>
       <c r="H39" s="2" t="s">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="I39" s="10"/>
       <c r="J39" s="10"/>
@@ -5288,12 +5334,12 @@
       <c r="Y39" s="10"/>
       <c r="Z39" s="10"/>
     </row>
-    <row r="40" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
-        <v>80</v>
+    <row r="40" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A40" s="11" t="s">
+        <v>78</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>81</v>
+      <c r="B40" s="11" t="s">
+        <v>79</v>
       </c>
       <c r="C40" s="9"/>
       <c r="D40" s="2"/>
@@ -5303,7 +5349,7 @@
         <v>14</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I40" s="10"/>
       <c r="J40" s="10"/>
@@ -5325,17 +5371,21 @@
       <c r="Z40" s="10"/>
     </row>
     <row r="41" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="11"/>
-      <c r="B41" s="11" t="s">
-        <v>82</v>
+      <c r="A41" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="2"/>
       <c r="E41" s="9"/>
       <c r="F41" s="2"/>
-      <c r="G41" s="9"/>
+      <c r="G41" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="H41" s="2" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="I41" s="10"/>
       <c r="J41" s="10"/>
@@ -5356,22 +5406,18 @@
       <c r="Y41" s="10"/>
       <c r="Z41" s="10"/>
     </row>
-    <row r="42" spans="1:26" ht="93" x14ac:dyDescent="0.35">
-      <c r="A42" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>84</v>
+    <row r="42" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A42" s="11"/>
+      <c r="B42" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="C42" s="9"/>
       <c r="D42" s="2"/>
       <c r="E42" s="9"/>
       <c r="F42" s="2"/>
-      <c r="G42" s="9" t="s">
-        <v>14</v>
-      </c>
+      <c r="G42" s="9"/>
       <c r="H42" s="2" t="s">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
@@ -5392,10 +5438,12 @@
       <c r="Y42" s="10"/>
       <c r="Z42" s="10"/>
     </row>
-    <row r="43" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A43" s="11"/>
-      <c r="B43" s="11" t="s">
-        <v>85</v>
+    <row r="43" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="2"/>
@@ -5405,7 +5453,7 @@
         <v>14</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I43" s="10"/>
       <c r="J43" s="10"/>
@@ -5426,22 +5474,20 @@
       <c r="Y43" s="10"/>
       <c r="Z43" s="10"/>
     </row>
-    <row r="44" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A44" s="11" t="s">
-        <v>86</v>
-      </c>
+    <row r="44" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="11"/>
       <c r="B44" s="11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="2"/>
       <c r="E44" s="9"/>
       <c r="F44" s="2"/>
       <c r="G44" s="9" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="I44" s="10"/>
       <c r="J44" s="10"/>
@@ -5462,12 +5508,12 @@
       <c r="Y44" s="10"/>
       <c r="Z44" s="10"/>
     </row>
-    <row r="45" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A45" s="11" t="s">
-        <v>88</v>
+    <row r="45" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A45" s="16" t="s">
+        <v>86</v>
       </c>
-      <c r="B45" s="11" t="s">
-        <v>89</v>
+      <c r="B45" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="2"/>
@@ -5477,7 +5523,7 @@
         <v>47</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I45" s="10"/>
       <c r="J45" s="10"/>
@@ -5498,22 +5544,24 @@
       <c r="Y45" s="10"/>
       <c r="Z45" s="10"/>
     </row>
-    <row r="46" spans="1:26" ht="124" x14ac:dyDescent="0.35">
-      <c r="A46" s="2" t="s">
-        <v>90</v>
+    <row r="46" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
+      <c r="A46" s="14" t="s">
+        <v>123</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>91</v>
+      <c r="B46" s="15" t="s">
+        <v>88</v>
       </c>
       <c r="C46" s="9"/>
       <c r="D46" s="2"/>
       <c r="E46" s="9"/>
-      <c r="F46" s="2"/>
+      <c r="F46" s="2" t="s">
+        <v>121</v>
+      </c>
       <c r="G46" s="9" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="I46" s="10"/>
       <c r="J46" s="10"/>
@@ -5534,21 +5582,17 @@
       <c r="Y46" s="10"/>
       <c r="Z46" s="10"/>
     </row>
-    <row r="47" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2" t="s">
-        <v>92</v>
+    <row r="47" spans="1:26" ht="47" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A47" s="17"/>
+      <c r="B47" s="15" t="s">
+        <v>122</v>
       </c>
       <c r="C47" s="9"/>
       <c r="D47" s="2"/>
       <c r="E47" s="9"/>
       <c r="F47" s="2"/>
-      <c r="G47" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H47" s="2" t="s">
-        <v>105</v>
-      </c>
+      <c r="G47" s="9"/>
+      <c r="H47" s="2"/>
       <c r="I47" s="10"/>
       <c r="J47" s="10"/>
       <c r="K47" s="10"/>
@@ -5568,10 +5612,12 @@
       <c r="Y47" s="10"/>
       <c r="Z47" s="10"/>
     </row>
-    <row r="48" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A48" s="11"/>
-      <c r="B48" s="11" t="s">
-        <v>93</v>
+    <row r="48" spans="1:26" ht="124" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="C48" s="9"/>
       <c r="D48" s="2"/>
@@ -5581,7 +5627,7 @@
         <v>14</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I48" s="10"/>
       <c r="J48" s="10"/>
@@ -5602,12 +5648,10 @@
       <c r="Y48" s="10"/>
       <c r="Z48" s="10"/>
     </row>
-    <row r="49" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A49" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="B49" s="11" t="s">
-        <v>95</v>
+    <row r="49" spans="1:26" ht="62" x14ac:dyDescent="0.35">
+      <c r="A49" s="2"/>
+      <c r="B49" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="2"/>
@@ -5617,7 +5661,7 @@
         <v>14</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
@@ -5638,12 +5682,10 @@
       <c r="Y49" s="10"/>
       <c r="Z49" s="10"/>
     </row>
-    <row r="50" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A50" s="11" t="s">
-        <v>96</v>
-      </c>
+    <row r="50" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A50" s="11"/>
       <c r="B50" s="11" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="2"/>
@@ -5653,7 +5695,7 @@
         <v>14</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I50" s="10"/>
       <c r="J50" s="10"/>
@@ -5674,12 +5716,12 @@
       <c r="Y50" s="10"/>
       <c r="Z50" s="10"/>
     </row>
-    <row r="51" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A51" s="2" t="s">
-        <v>98</v>
+    <row r="51" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A51" s="11" t="s">
+        <v>93</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>99</v>
+      <c r="B51" s="11" t="s">
+        <v>94</v>
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="2"/>
@@ -5689,7 +5731,7 @@
         <v>14</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="10"/>
@@ -5710,10 +5752,12 @@
       <c r="Y51" s="10"/>
       <c r="Z51" s="10"/>
     </row>
-    <row r="52" spans="1:26" ht="93" x14ac:dyDescent="0.35">
-      <c r="A52" s="11"/>
+    <row r="52" spans="1:26" ht="47" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A52" s="11" t="s">
+        <v>95</v>
+      </c>
       <c r="B52" s="11" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C52" s="9"/>
       <c r="D52" s="2"/>
@@ -5723,7 +5767,7 @@
         <v>14</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="I52" s="10"/>
       <c r="J52" s="10"/>
@@ -5744,12 +5788,12 @@
       <c r="Y52" s="10"/>
       <c r="Z52" s="10"/>
     </row>
-    <row r="53" spans="1:26" ht="93" x14ac:dyDescent="0.35">
-      <c r="A53" s="11" t="s">
-        <v>101</v>
+    <row r="53" spans="1:26" ht="62" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
+        <v>97</v>
       </c>
-      <c r="B53" s="11" t="s">
-        <v>102</v>
+      <c r="B53" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="2"/>
@@ -5759,7 +5803,7 @@
         <v>14</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I53" s="10"/>
       <c r="J53" s="10"/>
@@ -5780,19 +5824,17 @@
       <c r="Y53" s="10"/>
       <c r="Z53" s="10"/>
     </row>
-    <row r="54" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A54" s="11" t="s">
-        <v>103</v>
-      </c>
+    <row r="54" spans="1:26" ht="93.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A54" s="11"/>
       <c r="B54" s="11" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C54" s="9"/>
       <c r="D54" s="2"/>
       <c r="E54" s="9"/>
       <c r="F54" s="2"/>
       <c r="G54" s="9" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>114</v>
@@ -5816,15 +5858,23 @@
       <c r="Y54" s="10"/>
       <c r="Z54" s="10"/>
     </row>
-    <row r="55" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
+    <row r="55" spans="1:26" ht="93.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A55" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>101</v>
+      </c>
       <c r="C55" s="9"/>
       <c r="D55" s="2"/>
       <c r="E55" s="9"/>
       <c r="F55" s="2"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
+      <c r="G55" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="I55" s="10"/>
       <c r="J55" s="10"/>
       <c r="K55" s="10"/>
@@ -5844,15 +5894,23 @@
       <c r="Y55" s="10"/>
       <c r="Z55" s="10"/>
     </row>
-    <row r="56" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
+    <row r="56" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A56" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>103</v>
+      </c>
       <c r="C56" s="9"/>
       <c r="D56" s="2"/>
       <c r="E56" s="9"/>
       <c r="F56" s="2"/>
-      <c r="G56" s="9"/>
-      <c r="H56" s="2"/>
+      <c r="G56" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>113</v>
+      </c>
       <c r="I56" s="10"/>
       <c r="J56" s="10"/>
       <c r="K56" s="10"/>
@@ -5872,15 +5930,19 @@
       <c r="Y56" s="10"/>
       <c r="Z56" s="10"/>
     </row>
-    <row r="57" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
+    <row r="57" spans="1:26" ht="62" x14ac:dyDescent="0.35">
+      <c r="A57" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>116</v>
+      </c>
       <c r="C57" s="9"/>
       <c r="D57" s="2"/>
       <c r="E57" s="9"/>
       <c r="F57" s="2"/>
-      <c r="G57" s="9"/>
-      <c r="H57" s="2"/>
+      <c r="G57" s="6"/>
+      <c r="H57" s="6"/>
       <c r="I57" s="10"/>
       <c r="J57" s="10"/>
       <c r="K57" s="10"/>
@@ -5900,9 +5962,13 @@
       <c r="Y57" s="10"/>
       <c r="Z57" s="10"/>
     </row>
-    <row r="58" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
+    <row r="58" spans="1:26" ht="62" x14ac:dyDescent="0.35">
+      <c r="A58" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>119</v>
+      </c>
       <c r="C58" s="9"/>
       <c r="D58" s="2"/>
       <c r="E58" s="9"/>
@@ -7328,19 +7394,15 @@
       <c r="Y108" s="10"/>
       <c r="Z108" s="10"/>
     </row>
-    <row r="109" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="9"/>
       <c r="D109" s="2"/>
       <c r="E109" s="9"/>
       <c r="F109" s="2"/>
-      <c r="G109" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H109" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G109" s="9"/>
+      <c r="H109" s="2"/>
       <c r="I109" s="10"/>
       <c r="J109" s="10"/>
       <c r="K109" s="10"/>
@@ -7388,15 +7450,19 @@
       <c r="Y110" s="10"/>
       <c r="Z110" s="10"/>
     </row>
-    <row r="111" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="9"/>
       <c r="D111" s="2"/>
       <c r="E111" s="9"/>
       <c r="F111" s="2"/>
-      <c r="G111" s="9"/>
-      <c r="H111" s="2"/>
+      <c r="G111" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H111" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I111" s="10"/>
       <c r="J111" s="10"/>
       <c r="K111" s="10"/>
@@ -8844,19 +8910,15 @@
       <c r="Y162" s="10"/>
       <c r="Z162" s="10"/>
     </row>
-    <row r="163" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
       <c r="C163" s="9"/>
       <c r="D163" s="2"/>
       <c r="E163" s="9"/>
       <c r="F163" s="2"/>
-      <c r="G163" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H163" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G163" s="9"/>
+      <c r="H163" s="2"/>
       <c r="I163" s="10"/>
       <c r="J163" s="10"/>
       <c r="K163" s="10"/>
@@ -8904,15 +8966,19 @@
       <c r="Y164" s="10"/>
       <c r="Z164" s="10"/>
     </row>
-    <row r="165" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="9"/>
       <c r="D165" s="2"/>
       <c r="E165" s="9"/>
       <c r="F165" s="2"/>
-      <c r="G165" s="9"/>
-      <c r="H165" s="2"/>
+      <c r="G165" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H165" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I165" s="10"/>
       <c r="J165" s="10"/>
       <c r="K165" s="10"/>
@@ -10360,19 +10426,15 @@
       <c r="Y216" s="10"/>
       <c r="Z216" s="10"/>
     </row>
-    <row r="217" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A217" s="2"/>
       <c r="B217" s="2"/>
       <c r="C217" s="9"/>
       <c r="D217" s="2"/>
       <c r="E217" s="9"/>
       <c r="F217" s="2"/>
-      <c r="G217" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H217" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G217" s="9"/>
+      <c r="H217" s="2"/>
       <c r="I217" s="10"/>
       <c r="J217" s="10"/>
       <c r="K217" s="10"/>
@@ -10420,15 +10482,19 @@
       <c r="Y218" s="10"/>
       <c r="Z218" s="10"/>
     </row>
-    <row r="219" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A219" s="2"/>
       <c r="B219" s="2"/>
       <c r="C219" s="9"/>
       <c r="D219" s="2"/>
       <c r="E219" s="9"/>
       <c r="F219" s="2"/>
-      <c r="G219" s="9"/>
-      <c r="H219" s="2"/>
+      <c r="G219" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H219" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I219" s="10"/>
       <c r="J219" s="10"/>
       <c r="K219" s="10"/>
@@ -11431,9 +11497,9 @@
     <row r="255" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A255" s="2"/>
       <c r="B255" s="2"/>
-      <c r="C255" s="2"/>
+      <c r="C255" s="9"/>
       <c r="D255" s="2"/>
-      <c r="E255" s="2"/>
+      <c r="E255" s="9"/>
       <c r="F255" s="2"/>
       <c r="G255" s="9"/>
       <c r="H255" s="2"/>
@@ -11459,9 +11525,9 @@
     <row r="256" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A256" s="2"/>
       <c r="B256" s="2"/>
-      <c r="C256" s="2"/>
+      <c r="C256" s="9"/>
       <c r="D256" s="2"/>
-      <c r="E256" s="2"/>
+      <c r="E256" s="9"/>
       <c r="F256" s="2"/>
       <c r="G256" s="9"/>
       <c r="H256" s="2"/>
@@ -11876,19 +11942,15 @@
       <c r="Y270" s="10"/>
       <c r="Z270" s="10"/>
     </row>
-    <row r="271" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A271" s="2"/>
       <c r="B271" s="2"/>
       <c r="C271" s="2"/>
       <c r="D271" s="2"/>
       <c r="E271" s="2"/>
       <c r="F271" s="2"/>
-      <c r="G271" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H271" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G271" s="9"/>
+      <c r="H271" s="2"/>
       <c r="I271" s="10"/>
       <c r="J271" s="10"/>
       <c r="K271" s="10"/>
@@ -11936,15 +11998,19 @@
       <c r="Y272" s="10"/>
       <c r="Z272" s="10"/>
     </row>
-    <row r="273" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A273" s="2"/>
       <c r="B273" s="2"/>
       <c r="C273" s="2"/>
       <c r="D273" s="2"/>
       <c r="E273" s="2"/>
       <c r="F273" s="2"/>
-      <c r="G273" s="9"/>
-      <c r="H273" s="2"/>
+      <c r="G273" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H273" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I273" s="10"/>
       <c r="J273" s="10"/>
       <c r="K273" s="10"/>
@@ -13392,19 +13458,15 @@
       <c r="Y324" s="10"/>
       <c r="Z324" s="10"/>
     </row>
-    <row r="325" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A325" s="2"/>
       <c r="B325" s="2"/>
       <c r="C325" s="2"/>
       <c r="D325" s="2"/>
       <c r="E325" s="2"/>
       <c r="F325" s="2"/>
-      <c r="G325" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H325" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G325" s="9"/>
+      <c r="H325" s="2"/>
       <c r="I325" s="10"/>
       <c r="J325" s="10"/>
       <c r="K325" s="10"/>
@@ -13452,15 +13514,19 @@
       <c r="Y326" s="10"/>
       <c r="Z326" s="10"/>
     </row>
-    <row r="327" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A327" s="2"/>
       <c r="B327" s="2"/>
       <c r="C327" s="2"/>
       <c r="D327" s="2"/>
       <c r="E327" s="2"/>
       <c r="F327" s="2"/>
-      <c r="G327" s="9"/>
-      <c r="H327" s="2"/>
+      <c r="G327" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H327" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I327" s="10"/>
       <c r="J327" s="10"/>
       <c r="K327" s="10"/>
@@ -14908,19 +14974,15 @@
       <c r="Y378" s="10"/>
       <c r="Z378" s="10"/>
     </row>
-    <row r="379" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A379" s="2"/>
       <c r="B379" s="2"/>
       <c r="C379" s="2"/>
       <c r="D379" s="2"/>
       <c r="E379" s="2"/>
       <c r="F379" s="2"/>
-      <c r="G379" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H379" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G379" s="9"/>
+      <c r="H379" s="2"/>
       <c r="I379" s="10"/>
       <c r="J379" s="10"/>
       <c r="K379" s="10"/>
@@ -14968,15 +15030,19 @@
       <c r="Y380" s="10"/>
       <c r="Z380" s="10"/>
     </row>
-    <row r="381" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A381" s="2"/>
       <c r="B381" s="2"/>
       <c r="C381" s="2"/>
       <c r="D381" s="2"/>
       <c r="E381" s="2"/>
       <c r="F381" s="2"/>
-      <c r="G381" s="9"/>
-      <c r="H381" s="2"/>
+      <c r="G381" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H381" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I381" s="10"/>
       <c r="J381" s="10"/>
       <c r="K381" s="10"/>
@@ -16424,19 +16490,15 @@
       <c r="Y432" s="10"/>
       <c r="Z432" s="10"/>
     </row>
-    <row r="433" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="433" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A433" s="2"/>
       <c r="B433" s="2"/>
       <c r="C433" s="2"/>
       <c r="D433" s="2"/>
       <c r="E433" s="2"/>
       <c r="F433" s="2"/>
-      <c r="G433" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H433" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G433" s="9"/>
+      <c r="H433" s="2"/>
       <c r="I433" s="10"/>
       <c r="J433" s="10"/>
       <c r="K433" s="10"/>
@@ -16484,15 +16546,19 @@
       <c r="Y434" s="10"/>
       <c r="Z434" s="10"/>
     </row>
-    <row r="435" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A435" s="2"/>
       <c r="B435" s="2"/>
       <c r="C435" s="2"/>
       <c r="D435" s="2"/>
       <c r="E435" s="2"/>
       <c r="F435" s="2"/>
-      <c r="G435" s="9"/>
-      <c r="H435" s="2"/>
+      <c r="G435" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H435" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I435" s="10"/>
       <c r="J435" s="10"/>
       <c r="K435" s="10"/>
@@ -17940,19 +18006,15 @@
       <c r="Y486" s="10"/>
       <c r="Z486" s="10"/>
     </row>
-    <row r="487" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="487" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A487" s="2"/>
       <c r="B487" s="2"/>
       <c r="C487" s="2"/>
       <c r="D487" s="2"/>
       <c r="E487" s="2"/>
       <c r="F487" s="2"/>
-      <c r="G487" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H487" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G487" s="9"/>
+      <c r="H487" s="2"/>
       <c r="I487" s="10"/>
       <c r="J487" s="10"/>
       <c r="K487" s="10"/>
@@ -18000,15 +18062,19 @@
       <c r="Y488" s="10"/>
       <c r="Z488" s="10"/>
     </row>
-    <row r="489" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="489" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A489" s="2"/>
       <c r="B489" s="2"/>
       <c r="C489" s="2"/>
       <c r="D489" s="2"/>
       <c r="E489" s="2"/>
       <c r="F489" s="2"/>
-      <c r="G489" s="9"/>
-      <c r="H489" s="2"/>
+      <c r="G489" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H489" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I489" s="10"/>
       <c r="J489" s="10"/>
       <c r="K489" s="10"/>
@@ -19456,19 +19522,15 @@
       <c r="Y540" s="10"/>
       <c r="Z540" s="10"/>
     </row>
-    <row r="541" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="541" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A541" s="2"/>
       <c r="B541" s="2"/>
       <c r="C541" s="2"/>
       <c r="D541" s="2"/>
       <c r="E541" s="2"/>
       <c r="F541" s="2"/>
-      <c r="G541" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H541" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G541" s="9"/>
+      <c r="H541" s="2"/>
       <c r="I541" s="10"/>
       <c r="J541" s="10"/>
       <c r="K541" s="10"/>
@@ -19516,15 +19578,19 @@
       <c r="Y542" s="10"/>
       <c r="Z542" s="10"/>
     </row>
-    <row r="543" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="543" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A543" s="2"/>
       <c r="B543" s="2"/>
       <c r="C543" s="2"/>
       <c r="D543" s="2"/>
       <c r="E543" s="2"/>
       <c r="F543" s="2"/>
-      <c r="G543" s="9"/>
-      <c r="H543" s="2"/>
+      <c r="G543" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H543" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I543" s="10"/>
       <c r="J543" s="10"/>
       <c r="K543" s="10"/>
@@ -20972,19 +21038,15 @@
       <c r="Y594" s="10"/>
       <c r="Z594" s="10"/>
     </row>
-    <row r="595" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="595" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A595" s="2"/>
       <c r="B595" s="2"/>
       <c r="C595" s="2"/>
       <c r="D595" s="2"/>
       <c r="E595" s="2"/>
       <c r="F595" s="2"/>
-      <c r="G595" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H595" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G595" s="9"/>
+      <c r="H595" s="2"/>
       <c r="I595" s="10"/>
       <c r="J595" s="10"/>
       <c r="K595" s="10"/>
@@ -21032,15 +21094,19 @@
       <c r="Y596" s="10"/>
       <c r="Z596" s="10"/>
     </row>
-    <row r="597" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="597" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A597" s="2"/>
       <c r="B597" s="2"/>
       <c r="C597" s="2"/>
       <c r="D597" s="2"/>
       <c r="E597" s="2"/>
       <c r="F597" s="2"/>
-      <c r="G597" s="9"/>
-      <c r="H597" s="2"/>
+      <c r="G597" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H597" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I597" s="10"/>
       <c r="J597" s="10"/>
       <c r="K597" s="10"/>
@@ -22488,19 +22554,15 @@
       <c r="Y648" s="10"/>
       <c r="Z648" s="10"/>
     </row>
-    <row r="649" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="649" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A649" s="2"/>
       <c r="B649" s="2"/>
       <c r="C649" s="2"/>
       <c r="D649" s="2"/>
       <c r="E649" s="2"/>
       <c r="F649" s="2"/>
-      <c r="G649" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H649" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G649" s="9"/>
+      <c r="H649" s="2"/>
       <c r="I649" s="10"/>
       <c r="J649" s="10"/>
       <c r="K649" s="10"/>
@@ -22548,15 +22610,19 @@
       <c r="Y650" s="10"/>
       <c r="Z650" s="10"/>
     </row>
-    <row r="651" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="651" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A651" s="2"/>
       <c r="B651" s="2"/>
       <c r="C651" s="2"/>
       <c r="D651" s="2"/>
       <c r="E651" s="2"/>
       <c r="F651" s="2"/>
-      <c r="G651" s="9"/>
-      <c r="H651" s="2"/>
+      <c r="G651" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H651" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I651" s="10"/>
       <c r="J651" s="10"/>
       <c r="K651" s="10"/>
@@ -24004,19 +24070,15 @@
       <c r="Y702" s="10"/>
       <c r="Z702" s="10"/>
     </row>
-    <row r="703" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="703" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A703" s="2"/>
       <c r="B703" s="2"/>
       <c r="C703" s="2"/>
       <c r="D703" s="2"/>
       <c r="E703" s="2"/>
       <c r="F703" s="2"/>
-      <c r="G703" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H703" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G703" s="9"/>
+      <c r="H703" s="2"/>
       <c r="I703" s="10"/>
       <c r="J703" s="10"/>
       <c r="K703" s="10"/>
@@ -24064,15 +24126,19 @@
       <c r="Y704" s="10"/>
       <c r="Z704" s="10"/>
     </row>
-    <row r="705" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="705" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A705" s="2"/>
       <c r="B705" s="2"/>
       <c r="C705" s="2"/>
       <c r="D705" s="2"/>
       <c r="E705" s="2"/>
       <c r="F705" s="2"/>
-      <c r="G705" s="9"/>
-      <c r="H705" s="2"/>
+      <c r="G705" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H705" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I705" s="10"/>
       <c r="J705" s="10"/>
       <c r="K705" s="10"/>
@@ -25520,19 +25586,15 @@
       <c r="Y756" s="10"/>
       <c r="Z756" s="10"/>
     </row>
-    <row r="757" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="757" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A757" s="2"/>
       <c r="B757" s="2"/>
       <c r="C757" s="2"/>
       <c r="D757" s="2"/>
       <c r="E757" s="2"/>
       <c r="F757" s="2"/>
-      <c r="G757" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H757" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G757" s="9"/>
+      <c r="H757" s="2"/>
       <c r="I757" s="10"/>
       <c r="J757" s="10"/>
       <c r="K757" s="10"/>
@@ -25580,15 +25642,19 @@
       <c r="Y758" s="10"/>
       <c r="Z758" s="10"/>
     </row>
-    <row r="759" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="759" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A759" s="2"/>
       <c r="B759" s="2"/>
       <c r="C759" s="2"/>
       <c r="D759" s="2"/>
       <c r="E759" s="2"/>
       <c r="F759" s="2"/>
-      <c r="G759" s="9"/>
-      <c r="H759" s="2"/>
+      <c r="G759" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H759" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I759" s="10"/>
       <c r="J759" s="10"/>
       <c r="K759" s="10"/>
@@ -27036,19 +27102,15 @@
       <c r="Y810" s="10"/>
       <c r="Z810" s="10"/>
     </row>
-    <row r="811" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="811" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A811" s="2"/>
       <c r="B811" s="2"/>
       <c r="C811" s="2"/>
       <c r="D811" s="2"/>
       <c r="E811" s="2"/>
       <c r="F811" s="2"/>
-      <c r="G811" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H811" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G811" s="9"/>
+      <c r="H811" s="2"/>
       <c r="I811" s="10"/>
       <c r="J811" s="10"/>
       <c r="K811" s="10"/>
@@ -27096,15 +27158,19 @@
       <c r="Y812" s="10"/>
       <c r="Z812" s="10"/>
     </row>
-    <row r="813" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="813" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A813" s="2"/>
       <c r="B813" s="2"/>
       <c r="C813" s="2"/>
       <c r="D813" s="2"/>
       <c r="E813" s="2"/>
       <c r="F813" s="2"/>
-      <c r="G813" s="9"/>
-      <c r="H813" s="2"/>
+      <c r="G813" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H813" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I813" s="10"/>
       <c r="J813" s="10"/>
       <c r="K813" s="10"/>
@@ -28552,19 +28618,15 @@
       <c r="Y864" s="10"/>
       <c r="Z864" s="10"/>
     </row>
-    <row r="865" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="865" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A865" s="2"/>
       <c r="B865" s="2"/>
       <c r="C865" s="2"/>
       <c r="D865" s="2"/>
       <c r="E865" s="2"/>
       <c r="F865" s="2"/>
-      <c r="G865" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H865" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G865" s="9"/>
+      <c r="H865" s="2"/>
       <c r="I865" s="10"/>
       <c r="J865" s="10"/>
       <c r="K865" s="10"/>
@@ -28612,15 +28674,19 @@
       <c r="Y866" s="10"/>
       <c r="Z866" s="10"/>
     </row>
-    <row r="867" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="867" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A867" s="2"/>
       <c r="B867" s="2"/>
       <c r="C867" s="2"/>
       <c r="D867" s="2"/>
       <c r="E867" s="2"/>
       <c r="F867" s="2"/>
-      <c r="G867" s="9"/>
-      <c r="H867" s="2"/>
+      <c r="G867" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H867" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I867" s="10"/>
       <c r="J867" s="10"/>
       <c r="K867" s="10"/>
@@ -30068,19 +30134,15 @@
       <c r="Y918" s="10"/>
       <c r="Z918" s="10"/>
     </row>
-    <row r="919" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+    <row r="919" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A919" s="2"/>
       <c r="B919" s="2"/>
       <c r="C919" s="2"/>
       <c r="D919" s="2"/>
       <c r="E919" s="2"/>
       <c r="F919" s="2"/>
-      <c r="G919" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H919" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G919" s="9"/>
+      <c r="H919" s="2"/>
       <c r="I919" s="10"/>
       <c r="J919" s="10"/>
       <c r="K919" s="10"/>
@@ -30128,15 +30190,19 @@
       <c r="Y920" s="10"/>
       <c r="Z920" s="10"/>
     </row>
-    <row r="921" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="921" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A921" s="2"/>
       <c r="B921" s="2"/>
       <c r="C921" s="2"/>
       <c r="D921" s="2"/>
       <c r="E921" s="2"/>
       <c r="F921" s="2"/>
-      <c r="G921" s="9"/>
-      <c r="H921" s="2"/>
+      <c r="G921" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H921" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I921" s="10"/>
       <c r="J921" s="10"/>
       <c r="K921" s="10"/>
@@ -31591,8 +31657,8 @@
       <c r="D973" s="2"/>
       <c r="E973" s="2"/>
       <c r="F973" s="2"/>
-      <c r="G973" s="10"/>
-      <c r="H973" s="10"/>
+      <c r="G973" s="9"/>
+      <c r="H973" s="2"/>
       <c r="I973" s="10"/>
       <c r="J973" s="10"/>
       <c r="K973" s="10"/>
@@ -31619,8 +31685,8 @@
       <c r="D974" s="2"/>
       <c r="E974" s="2"/>
       <c r="F974" s="2"/>
-      <c r="G974" s="10"/>
-      <c r="H974" s="10"/>
+      <c r="G974" s="9"/>
+      <c r="H974" s="2"/>
       <c r="I974" s="10"/>
       <c r="J974" s="10"/>
       <c r="K974" s="10"/>
@@ -32368,9 +32434,65 @@
       <c r="Y1000" s="10"/>
       <c r="Z1000" s="10"/>
     </row>
+    <row r="1001" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1001" s="2"/>
+      <c r="B1001" s="2"/>
+      <c r="C1001" s="2"/>
+      <c r="D1001" s="2"/>
+      <c r="E1001" s="2"/>
+      <c r="F1001" s="2"/>
+      <c r="G1001" s="10"/>
+      <c r="H1001" s="10"/>
+      <c r="I1001" s="10"/>
+      <c r="J1001" s="10"/>
+      <c r="K1001" s="10"/>
+      <c r="L1001" s="10"/>
+      <c r="M1001" s="10"/>
+      <c r="N1001" s="10"/>
+      <c r="O1001" s="10"/>
+      <c r="P1001" s="10"/>
+      <c r="Q1001" s="10"/>
+      <c r="R1001" s="10"/>
+      <c r="S1001" s="10"/>
+      <c r="T1001" s="10"/>
+      <c r="U1001" s="10"/>
+      <c r="V1001" s="10"/>
+      <c r="W1001" s="10"/>
+      <c r="X1001" s="10"/>
+      <c r="Y1001" s="10"/>
+      <c r="Z1001" s="10"/>
+    </row>
+    <row r="1002" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1002" s="2"/>
+      <c r="B1002" s="2"/>
+      <c r="C1002" s="2"/>
+      <c r="D1002" s="2"/>
+      <c r="E1002" s="2"/>
+      <c r="F1002" s="2"/>
+      <c r="G1002" s="10"/>
+      <c r="H1002" s="10"/>
+      <c r="I1002" s="10"/>
+      <c r="J1002" s="10"/>
+      <c r="K1002" s="10"/>
+      <c r="L1002" s="10"/>
+      <c r="M1002" s="10"/>
+      <c r="N1002" s="10"/>
+      <c r="O1002" s="10"/>
+      <c r="P1002" s="10"/>
+      <c r="Q1002" s="10"/>
+      <c r="R1002" s="10"/>
+      <c r="S1002" s="10"/>
+      <c r="T1002" s="10"/>
+      <c r="U1002" s="10"/>
+      <c r="V1002" s="10"/>
+      <c r="W1002" s="10"/>
+      <c r="X1002" s="10"/>
+      <c r="Y1002" s="10"/>
+      <c r="Z1002" s="10"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G54 C2:C1000 E2:E1000 G56:G108 G110:G162 G164:G216 G218:G270 G272:G324 G326:G378 G380:G432 G434:G486 G488:G540 G542:G594 G596:G648 G650:G702 G704:G756 G758:G810 G812:G864 G866:G918 G920:G972">
+  <conditionalFormatting sqref="G2:G56 C2:C1002 E2:E1002 G58:G110 G112:G164 G166:G218 G220:G272 G274:G326 G328:G380 G382:G434 G436:G488 G490:G542 G544:G596 G598:G650 G652:G704 G706:G758 G760:G812 G814:G866 G868:G920 G922:G974">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
@@ -32378,7 +32500,7 @@
       <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D1000 F2:F1000 H56:H108 H110:H162 H164:H216 H218:H270 H272:H324 H326:H378 H380:H432 H434:H486 H488:H540 H542:H594 H596:H648 H650:H702 H704:H756 H758:H810 H812:H864 H866:H918 H920:H972 H2:H54">
+  <conditionalFormatting sqref="H2:H56 D2:D1002 F2:F1002 H58:H110 H112:H164 H166:H218 H220:H272 H274:H326 H328:H380 H382:H434 H436:H488 H490:H542 H544:H596 H598:H650 H652:H704 H706:H758 H760:H812 H814:H866 H868:H920 H922:H974">
     <cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
       <formula>AND(ISBLANK(D2),C2="Pass")</formula>
     </cfRule>
@@ -32386,8 +32508,8 @@
       <formula>AND(ISBLANK(D2),C2="Fail")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G54 G56:G108 G110:G162 G164:G216 G218:G270 G272:G324 G326:G378 G380:G432 G434:G486 G488:G540 C2:C582 E2:E582 G542:G594 G596:G648 G650:G702 G704:G756 G758:G810 G812:G864 G866:G918 G920:G972" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G56 G58:G110 G112:G164 G166:G218 G220:G272 G274:G326 G328:G380 G382:G434 G436:G488 G490:G542 C2:C584 E2:E584 G544:G596 G598:G650 G652:G704 G706:G758 G760:G812 G814:G866 G868:G920 G922:G974" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update ATP for phase 3
</commit_message>
<xml_diff>
--- a/etc/Acceptance Test Plan.xlsx
+++ b/etc/Acceptance Test Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phine\OneDrive\code2\swen\project\team-project-2251-swen-261-05-2-goated\etc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD2EE67F-08D5-4A77-A06D-A8B6F5374D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F98D5CC-7550-465C-9B5A-6324C60C7FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Test Plan" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Plan'!$G$1:$G$1002</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Plan'!$G$1:$G$1003</definedName>
   </definedNames>
   <calcPr calcId="0" concurrentCalc="0"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="139">
   <si>
     <t>Instructions</t>
   </si>
@@ -339,9 +339,6 @@
     <t>As a Manager I want to List people who have donated recently so that people can be thanked, and people can be encouraged to donate (so that their name appears).</t>
   </si>
   <si>
-    <t>**Given** a user is logged in **when** I access the home page **then** I can see a more elaborate list of 'thank you's (all of the 'thank you's).</t>
-  </si>
-  <si>
     <t>As a User I want to see the home/landing page so that I can initially access the app.</t>
   </si>
   <si>
@@ -406,6 +403,54 @@
   </si>
   <si>
     <t>As a user I want to have all tabs located in a navigation menu so that the website looks better.</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. However, it lets you change your password to what it already was, and the answer shows up in plaintext.</t>
+  </si>
+  <si>
+    <t>**Given** a user is logged in **when** I access the thanks page **then** I can see a more elaborate list of 'thank you's (all of the 'thank you's).</t>
+  </si>
+  <si>
+    <t>MM, CM 11/6/2025 (editor's note: the AC technically failed as it was written down incorrectly, however the testers did not notice this)</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. It also allows you to filter this pie chart</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. It only displays the buttons which your account has access to. (For Managers, this is everything but Basket. For Users, this is everything but Users.)</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. Read previous.</t>
+  </si>
+  <si>
+    <t>Given that I am logged in, I should see a button to log out of my account on the sidebar.</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. See previous</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. Also not case-sensitive.</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. In specific, there will be an alert stating that the user is not authorized to do this. This currently only applies to adding a need to a basket or checking a basket out.</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. This was tested by manually setting the timeout for 10 seconds. There is no alert that this happens, it will simply log you out when trying to switch pages after this hour.</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. This happens in the "Leaderboard" tab, where the top few users contributing the most needs are listed. n is given by the user.</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. If no users have contributed any needs, it will not display any users on this leaderboard.</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. This happens in the "Thanks" tab, where sets of 30 completed needs are listed, paged.</t>
+  </si>
+  <si>
+    <t>AF, 11/10/2025. If no needs have been satisfied, the "Thanks" tab and  home page preview are empty.</t>
   </si>
 </sst>
 </file>
@@ -502,7 +547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -540,14 +585,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3834,7 +3885,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z1002"/>
+  <dimension ref="A1:Z1003"/>
   <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -3905,13 +3956,17 @@
       <c r="D2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="2"/>
+      <c r="E2" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G2" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I2" s="10"/>
       <c r="J2" s="10"/>
@@ -3943,13 +3998,17 @@
       <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="9"/>
-      <c r="F3" s="2"/>
+      <c r="E3" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G3" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I3" s="10"/>
       <c r="J3" s="10"/>
@@ -3983,13 +4042,17 @@
       <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="9"/>
-      <c r="F4" s="2"/>
+      <c r="E4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G4" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I4" s="10"/>
       <c r="J4" s="10"/>
@@ -4023,13 +4086,17 @@
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="9"/>
-      <c r="F5" s="2"/>
+      <c r="E5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G5" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
@@ -4061,13 +4128,17 @@
       <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="2"/>
+      <c r="E6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G6" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
@@ -4101,13 +4172,17 @@
       <c r="D7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="9"/>
-      <c r="F7" s="2"/>
+      <c r="E7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G7" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
@@ -4141,13 +4216,17 @@
       <c r="D8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="2"/>
+      <c r="E8" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>131</v>
+      </c>
       <c r="G8" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
@@ -4179,13 +4258,17 @@
       <c r="D9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="2"/>
+      <c r="E9" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G9" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
@@ -4219,13 +4302,17 @@
       <c r="D10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="2"/>
+      <c r="E10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G10" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
@@ -4257,13 +4344,17 @@
       <c r="D11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="2"/>
+      <c r="E11" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G11" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
@@ -4295,13 +4386,17 @@
       <c r="D12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="2"/>
+      <c r="E12" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G12" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
@@ -4335,13 +4430,17 @@
       <c r="D13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="2"/>
+      <c r="E13" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G13" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
@@ -4375,13 +4474,17 @@
       <c r="D14" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="2"/>
+      <c r="E14" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G14" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
@@ -4413,13 +4516,17 @@
       <c r="D15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="2"/>
+      <c r="E15" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G15" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I15" s="10"/>
       <c r="J15" s="10"/>
@@ -4453,13 +4560,17 @@
       <c r="D16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="9"/>
-      <c r="F16" s="2"/>
+      <c r="E16" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G16" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
@@ -4491,13 +4602,17 @@
       <c r="D17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="9"/>
-      <c r="F17" s="2"/>
+      <c r="E17" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G17" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
@@ -4531,13 +4646,17 @@
       <c r="D18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="9"/>
-      <c r="F18" s="2"/>
+      <c r="E18" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G18" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I18" s="10"/>
       <c r="J18" s="10"/>
@@ -4569,13 +4688,17 @@
       <c r="D19" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="9"/>
-      <c r="F19" s="2"/>
+      <c r="E19" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G19" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I19" s="10"/>
       <c r="J19" s="10"/>
@@ -4607,13 +4730,17 @@
       <c r="D20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="9"/>
-      <c r="F20" s="2"/>
+      <c r="E20" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G20" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I20" s="10"/>
       <c r="J20" s="10"/>
@@ -4647,13 +4774,17 @@
       <c r="D21" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E21" s="9"/>
-      <c r="F21" s="2"/>
+      <c r="E21" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G21" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I21" s="10"/>
       <c r="J21" s="10"/>
@@ -4685,13 +4816,17 @@
       <c r="D22" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="9"/>
-      <c r="F22" s="2"/>
+      <c r="E22" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G22" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I22" s="10"/>
       <c r="J22" s="10"/>
@@ -4723,13 +4858,17 @@
       <c r="D23" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="9"/>
-      <c r="F23" s="2"/>
+      <c r="E23" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G23" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I23" s="10"/>
       <c r="J23" s="10"/>
@@ -4763,13 +4902,17 @@
       <c r="D24" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E24" s="9"/>
-      <c r="F24" s="2"/>
+      <c r="E24" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G24" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I24" s="10"/>
       <c r="J24" s="10"/>
@@ -4801,13 +4944,17 @@
       <c r="D25" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E25" s="9"/>
-      <c r="F25" s="2"/>
+      <c r="E25" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G25" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I25" s="10"/>
       <c r="J25" s="10"/>
@@ -4841,13 +4988,17 @@
       <c r="D26" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="9"/>
-      <c r="F26" s="2"/>
+      <c r="E26" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G26" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I26" s="10"/>
       <c r="J26" s="10"/>
@@ -4879,13 +5030,17 @@
       <c r="D27" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E27" s="9"/>
-      <c r="F27" s="2"/>
+      <c r="E27" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>129</v>
+      </c>
       <c r="G27" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I27" s="10"/>
       <c r="J27" s="10"/>
@@ -4919,13 +5074,17 @@
       <c r="D28" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E28" s="9"/>
-      <c r="F28" s="2"/>
+      <c r="E28" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G28" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I28" s="10"/>
       <c r="J28" s="10"/>
@@ -4947,8 +5106,8 @@
       <c r="Z28" s="10"/>
     </row>
     <row r="29" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="15"/>
-      <c r="B29" s="15" t="s">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C29" s="9" t="s">
@@ -4959,13 +5118,13 @@
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I29" s="10"/>
       <c r="J29" s="10"/>
@@ -4989,12 +5148,16 @@
     <row r="30" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="11"/>
       <c r="B30" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="2"/>
+      <c r="E30" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G30" s="9"/>
       <c r="H30" s="2"/>
       <c r="I30" s="10"/>
@@ -5016,11 +5179,11 @@
       <c r="Y30" s="10"/>
       <c r="Z30" s="10"/>
     </row>
-    <row r="31" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="12" t="s">
+    <row r="31" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="18" t="s">
         <v>64</v>
       </c>
       <c r="C31" s="9" t="s">
@@ -5029,13 +5192,14 @@
       <c r="D31" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E31" s="9"/>
-      <c r="F31" s="2"/>
+      <c r="F31" s="2" t="s">
+        <v>120</v>
+      </c>
       <c r="G31" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I31" s="10"/>
       <c r="J31" s="10"/>
@@ -5056,23 +5220,21 @@
       <c r="Y31" s="10"/>
       <c r="Z31" s="10"/>
     </row>
-    <row r="32" spans="1:26" ht="93" x14ac:dyDescent="0.35">
-      <c r="A32" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>66</v>
+    <row r="32" spans="1:26" ht="47" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="19"/>
+      <c r="B32" s="18" t="s">
+        <v>130</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="9" t="s">
+      <c r="E32" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H32" s="2" t="s">
-        <v>104</v>
-      </c>
+      <c r="F32" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G32" s="9"/>
+      <c r="H32" s="2"/>
       <c r="I32" s="10"/>
       <c r="J32" s="10"/>
       <c r="K32" s="10"/>
@@ -5092,20 +5254,26 @@
       <c r="Y32" s="10"/>
       <c r="Z32" s="10"/>
     </row>
-    <row r="33" spans="1:26" ht="93.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="12"/>
-      <c r="B33" s="11" t="s">
-        <v>67</v>
+    <row r="33" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+      <c r="A33" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>66</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="2"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="2"/>
+      <c r="E33" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>135</v>
+      </c>
       <c r="G33" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I33" s="10"/>
       <c r="J33" s="10"/>
@@ -5126,22 +5294,24 @@
       <c r="Y33" s="10"/>
       <c r="Z33" s="10"/>
     </row>
-    <row r="34" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A34" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>69</v>
+    <row r="34" spans="1:26" ht="93.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="12"/>
+      <c r="B34" s="11" t="s">
+        <v>67</v>
       </c>
       <c r="C34" s="9"/>
       <c r="D34" s="2"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="2"/>
+      <c r="E34" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="G34" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I34" s="10"/>
       <c r="J34" s="10"/>
@@ -5162,20 +5332,26 @@
       <c r="Y34" s="10"/>
       <c r="Z34" s="10"/>
     </row>
-    <row r="35" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="11"/>
-      <c r="B35" s="11" t="s">
-        <v>70</v>
+    <row r="35" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>69</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="2"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="2"/>
+      <c r="E35" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G35" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I35" s="10"/>
       <c r="J35" s="10"/>
@@ -5196,22 +5372,24 @@
       <c r="Y35" s="10"/>
       <c r="Z35" s="10"/>
     </row>
-    <row r="36" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A36" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>72</v>
+    <row r="36" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="11"/>
+      <c r="B36" s="11" t="s">
+        <v>70</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="2"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="2"/>
+      <c r="E36" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G36" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I36" s="10"/>
       <c r="J36" s="10"/>
@@ -5232,20 +5410,26 @@
       <c r="Y36" s="10"/>
       <c r="Z36" s="10"/>
     </row>
-    <row r="37" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11" t="s">
-        <v>73</v>
+    <row r="37" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>72</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="2"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="2"/>
+      <c r="E37" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G37" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I37" s="10"/>
       <c r="J37" s="10"/>
@@ -5266,22 +5450,24 @@
       <c r="Y37" s="10"/>
       <c r="Z37" s="10"/>
     </row>
-    <row r="38" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A38" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>75</v>
+    <row r="38" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="11"/>
+      <c r="B38" s="11" t="s">
+        <v>73</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="2"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="2"/>
+      <c r="E38" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G38" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I38" s="10"/>
       <c r="J38" s="10"/>
@@ -5302,18 +5488,26 @@
       <c r="Y38" s="10"/>
       <c r="Z38" s="10"/>
     </row>
-    <row r="39" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="11"/>
-      <c r="B39" s="11" t="s">
-        <v>76</v>
+    <row r="39" spans="1:26" ht="62" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>75</v>
       </c>
       <c r="C39" s="9"/>
       <c r="D39" s="2"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="9"/>
+      <c r="E39" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="H39" s="2" t="s">
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="I39" s="10"/>
       <c r="J39" s="10"/>
@@ -5335,21 +5529,21 @@
       <c r="Z39" s="10"/>
     </row>
     <row r="40" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="11" t="s">
-        <v>78</v>
-      </c>
+      <c r="A40" s="11"/>
       <c r="B40" s="11" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C40" s="9"/>
       <c r="D40" s="2"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="9" t="s">
+      <c r="E40" s="9" t="s">
         <v>14</v>
       </c>
+      <c r="F40" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G40" s="9"/>
       <c r="H40" s="2" t="s">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="I40" s="10"/>
       <c r="J40" s="10"/>
@@ -5370,22 +5564,26 @@
       <c r="Y40" s="10"/>
       <c r="Z40" s="10"/>
     </row>
-    <row r="41" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>81</v>
+    <row r="41" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A41" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>79</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="2"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="2"/>
+      <c r="E41" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G41" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I41" s="10"/>
       <c r="J41" s="10"/>
@@ -5406,18 +5604,26 @@
       <c r="Y41" s="10"/>
       <c r="Z41" s="10"/>
     </row>
-    <row r="42" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11" t="s">
-        <v>82</v>
+    <row r="42" spans="1:26" ht="77.5" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="C42" s="9"/>
       <c r="D42" s="2"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="9"/>
+      <c r="E42" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="H42" s="2" t="s">
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
@@ -5438,22 +5644,22 @@
       <c r="Y42" s="10"/>
       <c r="Z42" s="10"/>
     </row>
-    <row r="43" spans="1:26" ht="93" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>84</v>
+    <row r="43" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A43" s="11"/>
+      <c r="B43" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="2"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="9" t="s">
+      <c r="E43" s="9" t="s">
         <v>14</v>
       </c>
+      <c r="F43" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G43" s="9"/>
       <c r="H43" s="2" t="s">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="I43" s="10"/>
       <c r="J43" s="10"/>
@@ -5474,20 +5680,26 @@
       <c r="Y43" s="10"/>
       <c r="Z43" s="10"/>
     </row>
-    <row r="44" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A44" s="11"/>
-      <c r="B44" s="11" t="s">
-        <v>85</v>
+    <row r="44" spans="1:26" ht="93" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="2"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="2"/>
+      <c r="E44" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G44" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I44" s="10"/>
       <c r="J44" s="10"/>
@@ -5508,22 +5720,24 @@
       <c r="Y44" s="10"/>
       <c r="Z44" s="10"/>
     </row>
-    <row r="45" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A45" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="B45" s="16" t="s">
-        <v>87</v>
+    <row r="45" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A45" s="11"/>
+      <c r="B45" s="11" t="s">
+        <v>85</v>
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="2"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="2"/>
+      <c r="E45" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>133</v>
+      </c>
       <c r="G45" s="9" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="I45" s="10"/>
       <c r="J45" s="10"/>
@@ -5544,24 +5758,26 @@
       <c r="Y45" s="10"/>
       <c r="Z45" s="10"/>
     </row>
-    <row r="46" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A46" s="14" t="s">
-        <v>123</v>
+    <row r="46" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A46" s="15" t="s">
+        <v>86</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C46" s="9"/>
       <c r="D46" s="2"/>
-      <c r="E46" s="9"/>
+      <c r="E46" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="F46" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>47</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I46" s="10"/>
       <c r="J46" s="10"/>
@@ -5582,17 +5798,25 @@
       <c r="Y46" s="10"/>
       <c r="Z46" s="10"/>
     </row>
-    <row r="47" spans="1:26" ht="47" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A47" s="17"/>
-      <c r="B47" s="15" t="s">
+    <row r="47" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
+      <c r="A47" s="14" t="s">
         <v>122</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="C47" s="9"/>
       <c r="D47" s="2"/>
       <c r="E47" s="9"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="9"/>
-      <c r="H47" s="2"/>
+      <c r="F47" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>111</v>
+      </c>
       <c r="I47" s="10"/>
       <c r="J47" s="10"/>
       <c r="K47" s="10"/>
@@ -5612,23 +5836,21 @@
       <c r="Y47" s="10"/>
       <c r="Z47" s="10"/>
     </row>
-    <row r="48" spans="1:26" ht="124" x14ac:dyDescent="0.35">
-      <c r="A48" s="2" t="s">
-        <v>89</v>
-      </c>
+    <row r="48" spans="1:26" ht="47" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A48" s="16"/>
       <c r="B48" s="2" t="s">
-        <v>90</v>
+        <v>121</v>
       </c>
       <c r="C48" s="9"/>
       <c r="D48" s="2"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="2"/>
-      <c r="G48" s="9" t="s">
+      <c r="E48" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H48" s="2" t="s">
-        <v>104</v>
-      </c>
+      <c r="F48" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="G48" s="9"/>
+      <c r="H48" s="2"/>
       <c r="I48" s="10"/>
       <c r="J48" s="10"/>
       <c r="K48" s="10"/>
@@ -5648,20 +5870,26 @@
       <c r="Y48" s="10"/>
       <c r="Z48" s="10"/>
     </row>
-    <row r="49" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A49" s="2"/>
+    <row r="49" spans="1:26" ht="124" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="B49" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="2"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="2"/>
+      <c r="E49" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G49" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
@@ -5682,20 +5910,24 @@
       <c r="Y49" s="10"/>
       <c r="Z49" s="10"/>
     </row>
-    <row r="50" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A50" s="11"/>
-      <c r="B50" s="11" t="s">
-        <v>92</v>
+    <row r="50" spans="1:26" ht="62" x14ac:dyDescent="0.35">
+      <c r="A50" s="2"/>
+      <c r="B50" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="2"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="2"/>
+      <c r="E50" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G50" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I50" s="10"/>
       <c r="J50" s="10"/>
@@ -5716,22 +5948,24 @@
       <c r="Y50" s="10"/>
       <c r="Z50" s="10"/>
     </row>
-    <row r="51" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A51" s="11" t="s">
-        <v>93</v>
-      </c>
+    <row r="51" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A51" s="11"/>
       <c r="B51" s="11" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="2"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="2"/>
+      <c r="E51" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G51" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="10"/>
@@ -5752,22 +5986,26 @@
       <c r="Y51" s="10"/>
       <c r="Z51" s="10"/>
     </row>
-    <row r="52" spans="1:26" ht="47" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C52" s="9"/>
       <c r="D52" s="2"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="2"/>
+      <c r="E52" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>132</v>
+      </c>
       <c r="G52" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I52" s="10"/>
       <c r="J52" s="10"/>
@@ -5788,22 +6026,26 @@
       <c r="Y52" s="10"/>
       <c r="Z52" s="10"/>
     </row>
-    <row r="53" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A53" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>98</v>
+    <row r="53" spans="1:26" ht="47" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A53" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>96</v>
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="2"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="2"/>
+      <c r="E53" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G53" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I53" s="10"/>
       <c r="J53" s="10"/>
@@ -5824,20 +6066,26 @@
       <c r="Y53" s="10"/>
       <c r="Z53" s="10"/>
     </row>
-    <row r="54" spans="1:26" ht="93.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A54" s="11"/>
-      <c r="B54" s="11" t="s">
-        <v>99</v>
+    <row r="54" spans="1:26" ht="62" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="C54" s="9"/>
       <c r="D54" s="2"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="2"/>
+      <c r="E54" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G54" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="I54" s="10"/>
       <c r="J54" s="10"/>
@@ -5859,21 +6107,23 @@
       <c r="Z54" s="10"/>
     </row>
     <row r="55" spans="1:26" ht="93.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A55" s="11" t="s">
-        <v>100</v>
-      </c>
+      <c r="A55" s="11"/>
       <c r="B55" s="11" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C55" s="9"/>
       <c r="D55" s="2"/>
-      <c r="E55" s="9"/>
-      <c r="F55" s="2"/>
+      <c r="E55" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="G55" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="I55" s="10"/>
       <c r="J55" s="10"/>
@@ -5894,22 +6144,26 @@
       <c r="Y55" s="10"/>
       <c r="Z55" s="10"/>
     </row>
-    <row r="56" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:26" ht="93.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="11" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="C56" s="9"/>
       <c r="D56" s="2"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="2"/>
+      <c r="E56" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="G56" s="9" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I56" s="10"/>
       <c r="J56" s="10"/>
@@ -5930,19 +6184,27 @@
       <c r="Y56" s="10"/>
       <c r="Z56" s="10"/>
     </row>
-    <row r="57" spans="1:26" ht="62" x14ac:dyDescent="0.35">
-      <c r="A57" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>116</v>
+    <row r="57" spans="1:26" ht="62.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A57" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>102</v>
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="2"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="6"/>
-      <c r="H57" s="6"/>
+      <c r="E57" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="I57" s="10"/>
       <c r="J57" s="10"/>
       <c r="K57" s="10"/>
@@ -5964,17 +6226,21 @@
     </row>
     <row r="58" spans="1:26" ht="62" x14ac:dyDescent="0.35">
       <c r="A58" s="14" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C58" s="9"/>
       <c r="D58" s="2"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="2"/>
-      <c r="G58" s="9"/>
-      <c r="H58" s="2"/>
+      <c r="E58" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G58" s="6"/>
+      <c r="H58" s="6"/>
       <c r="I58" s="10"/>
       <c r="J58" s="10"/>
       <c r="K58" s="10"/>
@@ -5994,13 +6260,21 @@
       <c r="Y58" s="10"/>
       <c r="Z58" s="10"/>
     </row>
-    <row r="59" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
+    <row r="59" spans="1:26" ht="62" x14ac:dyDescent="0.35">
+      <c r="A59" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>118</v>
+      </c>
       <c r="C59" s="9"/>
       <c r="D59" s="2"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="2"/>
+      <c r="E59" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>127</v>
+      </c>
       <c r="G59" s="9"/>
       <c r="H59" s="2"/>
       <c r="I59" s="10"/>
@@ -7450,19 +7724,15 @@
       <c r="Y110" s="10"/>
       <c r="Z110" s="10"/>
     </row>
-    <row r="111" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="9"/>
       <c r="D111" s="2"/>
       <c r="E111" s="9"/>
       <c r="F111" s="2"/>
-      <c r="G111" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H111" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G111" s="9"/>
+      <c r="H111" s="2"/>
       <c r="I111" s="10"/>
       <c r="J111" s="10"/>
       <c r="K111" s="10"/>
@@ -7482,15 +7752,19 @@
       <c r="Y111" s="10"/>
       <c r="Z111" s="10"/>
     </row>
-    <row r="112" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="9"/>
       <c r="D112" s="2"/>
       <c r="E112" s="9"/>
       <c r="F112" s="2"/>
-      <c r="G112" s="9"/>
-      <c r="H112" s="2"/>
+      <c r="G112" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H112" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I112" s="10"/>
       <c r="J112" s="10"/>
       <c r="K112" s="10"/>
@@ -8966,19 +9240,15 @@
       <c r="Y164" s="10"/>
       <c r="Z164" s="10"/>
     </row>
-    <row r="165" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="9"/>
       <c r="D165" s="2"/>
       <c r="E165" s="9"/>
       <c r="F165" s="2"/>
-      <c r="G165" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H165" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G165" s="9"/>
+      <c r="H165" s="2"/>
       <c r="I165" s="10"/>
       <c r="J165" s="10"/>
       <c r="K165" s="10"/>
@@ -8998,15 +9268,19 @@
       <c r="Y165" s="10"/>
       <c r="Z165" s="10"/>
     </row>
-    <row r="166" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
       <c r="C166" s="9"/>
       <c r="D166" s="2"/>
       <c r="E166" s="9"/>
       <c r="F166" s="2"/>
-      <c r="G166" s="9"/>
-      <c r="H166" s="2"/>
+      <c r="G166" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H166" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I166" s="10"/>
       <c r="J166" s="10"/>
       <c r="K166" s="10"/>
@@ -10482,19 +10756,15 @@
       <c r="Y218" s="10"/>
       <c r="Z218" s="10"/>
     </row>
-    <row r="219" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A219" s="2"/>
       <c r="B219" s="2"/>
       <c r="C219" s="9"/>
       <c r="D219" s="2"/>
       <c r="E219" s="9"/>
       <c r="F219" s="2"/>
-      <c r="G219" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H219" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G219" s="9"/>
+      <c r="H219" s="2"/>
       <c r="I219" s="10"/>
       <c r="J219" s="10"/>
       <c r="K219" s="10"/>
@@ -10514,15 +10784,19 @@
       <c r="Y219" s="10"/>
       <c r="Z219" s="10"/>
     </row>
-    <row r="220" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A220" s="2"/>
       <c r="B220" s="2"/>
       <c r="C220" s="9"/>
       <c r="D220" s="2"/>
       <c r="E220" s="9"/>
       <c r="F220" s="2"/>
-      <c r="G220" s="9"/>
-      <c r="H220" s="2"/>
+      <c r="G220" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H220" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I220" s="10"/>
       <c r="J220" s="10"/>
       <c r="K220" s="10"/>
@@ -11553,9 +11827,9 @@
     <row r="257" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A257" s="2"/>
       <c r="B257" s="2"/>
-      <c r="C257" s="2"/>
+      <c r="C257" s="9"/>
       <c r="D257" s="2"/>
-      <c r="E257" s="2"/>
+      <c r="E257" s="9"/>
       <c r="F257" s="2"/>
       <c r="G257" s="9"/>
       <c r="H257" s="2"/>
@@ -11998,19 +12272,15 @@
       <c r="Y272" s="10"/>
       <c r="Z272" s="10"/>
     </row>
-    <row r="273" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A273" s="2"/>
       <c r="B273" s="2"/>
       <c r="C273" s="2"/>
       <c r="D273" s="2"/>
       <c r="E273" s="2"/>
       <c r="F273" s="2"/>
-      <c r="G273" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H273" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G273" s="9"/>
+      <c r="H273" s="2"/>
       <c r="I273" s="10"/>
       <c r="J273" s="10"/>
       <c r="K273" s="10"/>
@@ -12030,15 +12300,19 @@
       <c r="Y273" s="10"/>
       <c r="Z273" s="10"/>
     </row>
-    <row r="274" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A274" s="2"/>
       <c r="B274" s="2"/>
       <c r="C274" s="2"/>
       <c r="D274" s="2"/>
       <c r="E274" s="2"/>
       <c r="F274" s="2"/>
-      <c r="G274" s="9"/>
-      <c r="H274" s="2"/>
+      <c r="G274" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H274" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I274" s="10"/>
       <c r="J274" s="10"/>
       <c r="K274" s="10"/>
@@ -13514,19 +13788,15 @@
       <c r="Y326" s="10"/>
       <c r="Z326" s="10"/>
     </row>
-    <row r="327" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A327" s="2"/>
       <c r="B327" s="2"/>
       <c r="C327" s="2"/>
       <c r="D327" s="2"/>
       <c r="E327" s="2"/>
       <c r="F327" s="2"/>
-      <c r="G327" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H327" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G327" s="9"/>
+      <c r="H327" s="2"/>
       <c r="I327" s="10"/>
       <c r="J327" s="10"/>
       <c r="K327" s="10"/>
@@ -13546,15 +13816,19 @@
       <c r="Y327" s="10"/>
       <c r="Z327" s="10"/>
     </row>
-    <row r="328" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A328" s="2"/>
       <c r="B328" s="2"/>
       <c r="C328" s="2"/>
       <c r="D328" s="2"/>
       <c r="E328" s="2"/>
       <c r="F328" s="2"/>
-      <c r="G328" s="9"/>
-      <c r="H328" s="2"/>
+      <c r="G328" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H328" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I328" s="10"/>
       <c r="J328" s="10"/>
       <c r="K328" s="10"/>
@@ -15030,19 +15304,15 @@
       <c r="Y380" s="10"/>
       <c r="Z380" s="10"/>
     </row>
-    <row r="381" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A381" s="2"/>
       <c r="B381" s="2"/>
       <c r="C381" s="2"/>
       <c r="D381" s="2"/>
       <c r="E381" s="2"/>
       <c r="F381" s="2"/>
-      <c r="G381" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H381" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G381" s="9"/>
+      <c r="H381" s="2"/>
       <c r="I381" s="10"/>
       <c r="J381" s="10"/>
       <c r="K381" s="10"/>
@@ -15062,15 +15332,19 @@
       <c r="Y381" s="10"/>
       <c r="Z381" s="10"/>
     </row>
-    <row r="382" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A382" s="2"/>
       <c r="B382" s="2"/>
       <c r="C382" s="2"/>
       <c r="D382" s="2"/>
       <c r="E382" s="2"/>
       <c r="F382" s="2"/>
-      <c r="G382" s="9"/>
-      <c r="H382" s="2"/>
+      <c r="G382" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H382" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I382" s="10"/>
       <c r="J382" s="10"/>
       <c r="K382" s="10"/>
@@ -16546,19 +16820,15 @@
       <c r="Y434" s="10"/>
       <c r="Z434" s="10"/>
     </row>
-    <row r="435" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="435" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A435" s="2"/>
       <c r="B435" s="2"/>
       <c r="C435" s="2"/>
       <c r="D435" s="2"/>
       <c r="E435" s="2"/>
       <c r="F435" s="2"/>
-      <c r="G435" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H435" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G435" s="9"/>
+      <c r="H435" s="2"/>
       <c r="I435" s="10"/>
       <c r="J435" s="10"/>
       <c r="K435" s="10"/>
@@ -16578,15 +16848,19 @@
       <c r="Y435" s="10"/>
       <c r="Z435" s="10"/>
     </row>
-    <row r="436" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="436" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A436" s="2"/>
       <c r="B436" s="2"/>
       <c r="C436" s="2"/>
       <c r="D436" s="2"/>
       <c r="E436" s="2"/>
       <c r="F436" s="2"/>
-      <c r="G436" s="9"/>
-      <c r="H436" s="2"/>
+      <c r="G436" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H436" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I436" s="10"/>
       <c r="J436" s="10"/>
       <c r="K436" s="10"/>
@@ -18062,19 +18336,15 @@
       <c r="Y488" s="10"/>
       <c r="Z488" s="10"/>
     </row>
-    <row r="489" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="489" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A489" s="2"/>
       <c r="B489" s="2"/>
       <c r="C489" s="2"/>
       <c r="D489" s="2"/>
       <c r="E489" s="2"/>
       <c r="F489" s="2"/>
-      <c r="G489" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H489" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G489" s="9"/>
+      <c r="H489" s="2"/>
       <c r="I489" s="10"/>
       <c r="J489" s="10"/>
       <c r="K489" s="10"/>
@@ -18094,15 +18364,19 @@
       <c r="Y489" s="10"/>
       <c r="Z489" s="10"/>
     </row>
-    <row r="490" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="490" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A490" s="2"/>
       <c r="B490" s="2"/>
       <c r="C490" s="2"/>
       <c r="D490" s="2"/>
       <c r="E490" s="2"/>
       <c r="F490" s="2"/>
-      <c r="G490" s="9"/>
-      <c r="H490" s="2"/>
+      <c r="G490" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H490" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I490" s="10"/>
       <c r="J490" s="10"/>
       <c r="K490" s="10"/>
@@ -19578,19 +19852,15 @@
       <c r="Y542" s="10"/>
       <c r="Z542" s="10"/>
     </row>
-    <row r="543" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="543" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A543" s="2"/>
       <c r="B543" s="2"/>
       <c r="C543" s="2"/>
       <c r="D543" s="2"/>
       <c r="E543" s="2"/>
       <c r="F543" s="2"/>
-      <c r="G543" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H543" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G543" s="9"/>
+      <c r="H543" s="2"/>
       <c r="I543" s="10"/>
       <c r="J543" s="10"/>
       <c r="K543" s="10"/>
@@ -19610,15 +19880,19 @@
       <c r="Y543" s="10"/>
       <c r="Z543" s="10"/>
     </row>
-    <row r="544" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="544" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A544" s="2"/>
       <c r="B544" s="2"/>
       <c r="C544" s="2"/>
       <c r="D544" s="2"/>
       <c r="E544" s="2"/>
       <c r="F544" s="2"/>
-      <c r="G544" s="9"/>
-      <c r="H544" s="2"/>
+      <c r="G544" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H544" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I544" s="10"/>
       <c r="J544" s="10"/>
       <c r="K544" s="10"/>
@@ -21094,19 +21368,15 @@
       <c r="Y596" s="10"/>
       <c r="Z596" s="10"/>
     </row>
-    <row r="597" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="597" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A597" s="2"/>
       <c r="B597" s="2"/>
       <c r="C597" s="2"/>
       <c r="D597" s="2"/>
       <c r="E597" s="2"/>
       <c r="F597" s="2"/>
-      <c r="G597" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H597" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G597" s="9"/>
+      <c r="H597" s="2"/>
       <c r="I597" s="10"/>
       <c r="J597" s="10"/>
       <c r="K597" s="10"/>
@@ -21126,15 +21396,19 @@
       <c r="Y597" s="10"/>
       <c r="Z597" s="10"/>
     </row>
-    <row r="598" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="598" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A598" s="2"/>
       <c r="B598" s="2"/>
       <c r="C598" s="2"/>
       <c r="D598" s="2"/>
       <c r="E598" s="2"/>
       <c r="F598" s="2"/>
-      <c r="G598" s="9"/>
-      <c r="H598" s="2"/>
+      <c r="G598" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H598" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I598" s="10"/>
       <c r="J598" s="10"/>
       <c r="K598" s="10"/>
@@ -22610,19 +22884,15 @@
       <c r="Y650" s="10"/>
       <c r="Z650" s="10"/>
     </row>
-    <row r="651" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="651" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A651" s="2"/>
       <c r="B651" s="2"/>
       <c r="C651" s="2"/>
       <c r="D651" s="2"/>
       <c r="E651" s="2"/>
       <c r="F651" s="2"/>
-      <c r="G651" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H651" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G651" s="9"/>
+      <c r="H651" s="2"/>
       <c r="I651" s="10"/>
       <c r="J651" s="10"/>
       <c r="K651" s="10"/>
@@ -22642,15 +22912,19 @@
       <c r="Y651" s="10"/>
       <c r="Z651" s="10"/>
     </row>
-    <row r="652" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="652" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A652" s="2"/>
       <c r="B652" s="2"/>
       <c r="C652" s="2"/>
       <c r="D652" s="2"/>
       <c r="E652" s="2"/>
       <c r="F652" s="2"/>
-      <c r="G652" s="9"/>
-      <c r="H652" s="2"/>
+      <c r="G652" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H652" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I652" s="10"/>
       <c r="J652" s="10"/>
       <c r="K652" s="10"/>
@@ -24126,19 +24400,15 @@
       <c r="Y704" s="10"/>
       <c r="Z704" s="10"/>
     </row>
-    <row r="705" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="705" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A705" s="2"/>
       <c r="B705" s="2"/>
       <c r="C705" s="2"/>
       <c r="D705" s="2"/>
       <c r="E705" s="2"/>
       <c r="F705" s="2"/>
-      <c r="G705" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H705" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G705" s="9"/>
+      <c r="H705" s="2"/>
       <c r="I705" s="10"/>
       <c r="J705" s="10"/>
       <c r="K705" s="10"/>
@@ -24158,15 +24428,19 @@
       <c r="Y705" s="10"/>
       <c r="Z705" s="10"/>
     </row>
-    <row r="706" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="706" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A706" s="2"/>
       <c r="B706" s="2"/>
       <c r="C706" s="2"/>
       <c r="D706" s="2"/>
       <c r="E706" s="2"/>
       <c r="F706" s="2"/>
-      <c r="G706" s="9"/>
-      <c r="H706" s="2"/>
+      <c r="G706" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H706" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I706" s="10"/>
       <c r="J706" s="10"/>
       <c r="K706" s="10"/>
@@ -25642,19 +25916,15 @@
       <c r="Y758" s="10"/>
       <c r="Z758" s="10"/>
     </row>
-    <row r="759" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="759" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A759" s="2"/>
       <c r="B759" s="2"/>
       <c r="C759" s="2"/>
       <c r="D759" s="2"/>
       <c r="E759" s="2"/>
       <c r="F759" s="2"/>
-      <c r="G759" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H759" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G759" s="9"/>
+      <c r="H759" s="2"/>
       <c r="I759" s="10"/>
       <c r="J759" s="10"/>
       <c r="K759" s="10"/>
@@ -25674,15 +25944,19 @@
       <c r="Y759" s="10"/>
       <c r="Z759" s="10"/>
     </row>
-    <row r="760" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="760" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A760" s="2"/>
       <c r="B760" s="2"/>
       <c r="C760" s="2"/>
       <c r="D760" s="2"/>
       <c r="E760" s="2"/>
       <c r="F760" s="2"/>
-      <c r="G760" s="9"/>
-      <c r="H760" s="2"/>
+      <c r="G760" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H760" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I760" s="10"/>
       <c r="J760" s="10"/>
       <c r="K760" s="10"/>
@@ -27158,19 +27432,15 @@
       <c r="Y812" s="10"/>
       <c r="Z812" s="10"/>
     </row>
-    <row r="813" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="813" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A813" s="2"/>
       <c r="B813" s="2"/>
       <c r="C813" s="2"/>
       <c r="D813" s="2"/>
       <c r="E813" s="2"/>
       <c r="F813" s="2"/>
-      <c r="G813" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H813" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G813" s="9"/>
+      <c r="H813" s="2"/>
       <c r="I813" s="10"/>
       <c r="J813" s="10"/>
       <c r="K813" s="10"/>
@@ -27190,15 +27460,19 @@
       <c r="Y813" s="10"/>
       <c r="Z813" s="10"/>
     </row>
-    <row r="814" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="814" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A814" s="2"/>
       <c r="B814" s="2"/>
       <c r="C814" s="2"/>
       <c r="D814" s="2"/>
       <c r="E814" s="2"/>
       <c r="F814" s="2"/>
-      <c r="G814" s="9"/>
-      <c r="H814" s="2"/>
+      <c r="G814" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H814" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I814" s="10"/>
       <c r="J814" s="10"/>
       <c r="K814" s="10"/>
@@ -28674,19 +28948,15 @@
       <c r="Y866" s="10"/>
       <c r="Z866" s="10"/>
     </row>
-    <row r="867" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="867" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A867" s="2"/>
       <c r="B867" s="2"/>
       <c r="C867" s="2"/>
       <c r="D867" s="2"/>
       <c r="E867" s="2"/>
       <c r="F867" s="2"/>
-      <c r="G867" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H867" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G867" s="9"/>
+      <c r="H867" s="2"/>
       <c r="I867" s="10"/>
       <c r="J867" s="10"/>
       <c r="K867" s="10"/>
@@ -28706,15 +28976,19 @@
       <c r="Y867" s="10"/>
       <c r="Z867" s="10"/>
     </row>
-    <row r="868" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="868" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A868" s="2"/>
       <c r="B868" s="2"/>
       <c r="C868" s="2"/>
       <c r="D868" s="2"/>
       <c r="E868" s="2"/>
       <c r="F868" s="2"/>
-      <c r="G868" s="9"/>
-      <c r="H868" s="2"/>
+      <c r="G868" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H868" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I868" s="10"/>
       <c r="J868" s="10"/>
       <c r="K868" s="10"/>
@@ -30190,19 +30464,15 @@
       <c r="Y920" s="10"/>
       <c r="Z920" s="10"/>
     </row>
-    <row r="921" spans="1:26" ht="31" x14ac:dyDescent="0.35">
+    <row r="921" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A921" s="2"/>
       <c r="B921" s="2"/>
       <c r="C921" s="2"/>
       <c r="D921" s="2"/>
       <c r="E921" s="2"/>
       <c r="F921" s="2"/>
-      <c r="G921" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H921" s="6" t="s">
-        <v>9</v>
-      </c>
+      <c r="G921" s="9"/>
+      <c r="H921" s="2"/>
       <c r="I921" s="10"/>
       <c r="J921" s="10"/>
       <c r="K921" s="10"/>
@@ -30222,15 +30492,19 @@
       <c r="Y921" s="10"/>
       <c r="Z921" s="10"/>
     </row>
-    <row r="922" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="922" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A922" s="2"/>
       <c r="B922" s="2"/>
       <c r="C922" s="2"/>
       <c r="D922" s="2"/>
       <c r="E922" s="2"/>
       <c r="F922" s="2"/>
-      <c r="G922" s="9"/>
-      <c r="H922" s="2"/>
+      <c r="G922" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H922" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="I922" s="10"/>
       <c r="J922" s="10"/>
       <c r="K922" s="10"/>
@@ -31713,8 +31987,8 @@
       <c r="D975" s="2"/>
       <c r="E975" s="2"/>
       <c r="F975" s="2"/>
-      <c r="G975" s="10"/>
-      <c r="H975" s="10"/>
+      <c r="G975" s="9"/>
+      <c r="H975" s="2"/>
       <c r="I975" s="10"/>
       <c r="J975" s="10"/>
       <c r="K975" s="10"/>
@@ -32490,9 +32764,37 @@
       <c r="Y1002" s="10"/>
       <c r="Z1002" s="10"/>
     </row>
+    <row r="1003" spans="1:26" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1003" s="2"/>
+      <c r="B1003" s="2"/>
+      <c r="C1003" s="2"/>
+      <c r="D1003" s="2"/>
+      <c r="E1003" s="2"/>
+      <c r="F1003" s="2"/>
+      <c r="G1003" s="10"/>
+      <c r="H1003" s="10"/>
+      <c r="I1003" s="10"/>
+      <c r="J1003" s="10"/>
+      <c r="K1003" s="10"/>
+      <c r="L1003" s="10"/>
+      <c r="M1003" s="10"/>
+      <c r="N1003" s="10"/>
+      <c r="O1003" s="10"/>
+      <c r="P1003" s="10"/>
+      <c r="Q1003" s="10"/>
+      <c r="R1003" s="10"/>
+      <c r="S1003" s="10"/>
+      <c r="T1003" s="10"/>
+      <c r="U1003" s="10"/>
+      <c r="V1003" s="10"/>
+      <c r="W1003" s="10"/>
+      <c r="X1003" s="10"/>
+      <c r="Y1003" s="10"/>
+      <c r="Z1003" s="10"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G56 C2:C1002 E2:E1002 G58:G110 G112:G164 G166:G218 G220:G272 G274:G326 G328:G380 G382:G434 G436:G488 G490:G542 G544:G596 G598:G650 G652:G704 G706:G758 G760:G812 G814:G866 G868:G920 G922:G974">
+  <conditionalFormatting sqref="G2:G57 C2:C1003 G59:G111 G113:G165 G167:G219 G221:G273 G275:G327 G329:G381 G383:G435 G437:G489 G491:G543 G545:G597 G599:G651 G653:G705 G707:G759 G761:G813 G815:G867 G869:G921 G923:G975 E2:E30 E32:E1003">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
@@ -32500,7 +32802,7 @@
       <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H56 D2:D1002 F2:F1002 H58:H110 H112:H164 H166:H218 H220:H272 H274:H326 H328:H380 H382:H434 H436:H488 H490:H542 H544:H596 H598:H650 H652:H704 H706:H758 H760:H812 H814:H866 H868:H920 H922:H974">
+  <conditionalFormatting sqref="H2:H57 D2:D1003 H59:H111 H113:H165 H167:H219 H221:H273 H275:H327 H329:H381 H383:H435 H437:H489 H491:H543 H545:H597 H599:H651 H653:H705 H707:H759 H761:H813 H815:H867 H869:H921 H923:H975 F2:F1003">
     <cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
       <formula>AND(ISBLANK(D2),C2="Pass")</formula>
     </cfRule>
@@ -32508,8 +32810,8 @@
       <formula>AND(ISBLANK(D2),C2="Fail")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G56 G58:G110 G112:G164 G166:G218 G220:G272 G274:G326 G328:G380 G382:G434 G436:G488 G490:G542 C2:C584 E2:E584 G544:G596 G598:G650 G652:G704 G706:G758 G760:G812 G814:G866 G868:G920 G922:G974" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G57 G59:G111 G113:G165 G167:G219 G221:G273 G275:G327 G329:G381 G383:G435 G437:G489 G491:G543 C2:C585 G545:G597 G599:G651 G653:G705 G707:G759 G761:G813 G815:G867 G869:G921 G923:G975 E2:E30 E32:E585" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>